<commit_message>
feat: add label checking
</commit_message>
<xml_diff>
--- a/bert-tasks-class-label-mapping.xlsx
+++ b/bert-tasks-class-label-mapping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/longpham28/Documents/GitHub/ntcir19-pretrained-model-retrieval/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2BBF859-EDC9-F144-8A7A-083C30315C18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{082B7CBE-99E6-6F4E-8EBD-0E888DBC773C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25600" yWindow="600" windowWidth="25600" windowHeight="28200" xr2:uid="{0792540C-C5F0-BC4A-94C3-95ED34A20626}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="41120" windowHeight="25800" xr2:uid="{0792540C-C5F0-BC4A-94C3-95ED34A20626}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1036" uniqueCount="550">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1016" uniqueCount="530">
   <si>
     <t>cardiffnlp/tweet_eval@emoji</t>
   </si>
@@ -210,66 +210,6 @@
   </si>
   <si>
     <t>😜</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>7</t>
-  </si>
-  <si>
-    <t>8</t>
-  </si>
-  <si>
-    <t>9</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>11</t>
-  </si>
-  <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>13</t>
-  </si>
-  <si>
-    <t>14</t>
-  </si>
-  <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>16</t>
-  </si>
-  <si>
-    <t>17</t>
-  </si>
-  <si>
-    <t>18</t>
-  </si>
-  <si>
-    <t>19</t>
   </si>
   <si>
     <t>anger</t>
@@ -1824,11 +1764,14 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -2171,16 +2114,16 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>546</v>
+        <v>526</v>
       </c>
       <c r="B1" t="s">
-        <v>547</v>
+        <v>527</v>
       </c>
       <c r="C1" t="s">
-        <v>548</v>
+        <v>528</v>
       </c>
       <c r="D1" t="s">
-        <v>549</v>
+        <v>529</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -2190,8 +2133,8 @@
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" t="s">
-        <v>58</v>
+      <c r="C2" s="2">
+        <v>0</v>
       </c>
       <c r="D2" t="s">
         <v>38</v>
@@ -2204,8 +2147,8 @@
       <c r="B3" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C3" t="s">
-        <v>59</v>
+      <c r="C3" s="2">
+        <v>1</v>
       </c>
       <c r="D3" t="s">
         <v>39</v>
@@ -2218,8 +2161,8 @@
       <c r="B4" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C4" t="s">
-        <v>60</v>
+      <c r="C4" s="2">
+        <v>2</v>
       </c>
       <c r="D4" t="s">
         <v>40</v>
@@ -2232,8 +2175,8 @@
       <c r="B5" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C5" t="s">
-        <v>61</v>
+      <c r="C5" s="2">
+        <v>3</v>
       </c>
       <c r="D5" t="s">
         <v>41</v>
@@ -2246,8 +2189,8 @@
       <c r="B6" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C6" t="s">
-        <v>62</v>
+      <c r="C6" s="2">
+        <v>4</v>
       </c>
       <c r="D6" t="s">
         <v>42</v>
@@ -2260,8 +2203,8 @@
       <c r="B7" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C7" t="s">
-        <v>63</v>
+      <c r="C7" s="2">
+        <v>5</v>
       </c>
       <c r="D7" t="s">
         <v>43</v>
@@ -2274,8 +2217,8 @@
       <c r="B8" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C8" t="s">
-        <v>64</v>
+      <c r="C8" s="2">
+        <v>6</v>
       </c>
       <c r="D8" t="s">
         <v>44</v>
@@ -2288,8 +2231,8 @@
       <c r="B9" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C9" t="s">
-        <v>65</v>
+      <c r="C9" s="2">
+        <v>7</v>
       </c>
       <c r="D9" t="s">
         <v>45</v>
@@ -2302,8 +2245,8 @@
       <c r="B10" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C10" t="s">
-        <v>66</v>
+      <c r="C10" s="2">
+        <v>8</v>
       </c>
       <c r="D10" t="s">
         <v>46</v>
@@ -2316,8 +2259,8 @@
       <c r="B11" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C11" t="s">
-        <v>67</v>
+      <c r="C11" s="2">
+        <v>9</v>
       </c>
       <c r="D11" t="s">
         <v>47</v>
@@ -2330,8 +2273,8 @@
       <c r="B12" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C12" t="s">
-        <v>68</v>
+      <c r="C12" s="2">
+        <v>10</v>
       </c>
       <c r="D12" t="s">
         <v>48</v>
@@ -2344,8 +2287,8 @@
       <c r="B13" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C13" t="s">
-        <v>69</v>
+      <c r="C13" s="2">
+        <v>11</v>
       </c>
       <c r="D13" t="s">
         <v>49</v>
@@ -2358,8 +2301,8 @@
       <c r="B14" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C14" t="s">
-        <v>70</v>
+      <c r="C14" s="2">
+        <v>12</v>
       </c>
       <c r="D14" t="s">
         <v>50</v>
@@ -2372,8 +2315,8 @@
       <c r="B15" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C15" t="s">
-        <v>71</v>
+      <c r="C15" s="2">
+        <v>13</v>
       </c>
       <c r="D15" t="s">
         <v>51</v>
@@ -2386,8 +2329,8 @@
       <c r="B16" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C16" t="s">
-        <v>72</v>
+      <c r="C16" s="2">
+        <v>14</v>
       </c>
       <c r="D16" t="s">
         <v>52</v>
@@ -2400,8 +2343,8 @@
       <c r="B17" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C17" t="s">
-        <v>73</v>
+      <c r="C17" s="2">
+        <v>15</v>
       </c>
       <c r="D17" t="s">
         <v>53</v>
@@ -2414,8 +2357,8 @@
       <c r="B18" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C18" t="s">
-        <v>74</v>
+      <c r="C18" s="2">
+        <v>16</v>
       </c>
       <c r="D18" t="s">
         <v>54</v>
@@ -2428,8 +2371,8 @@
       <c r="B19" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C19" t="s">
-        <v>75</v>
+      <c r="C19" s="2">
+        <v>17</v>
       </c>
       <c r="D19" t="s">
         <v>55</v>
@@ -2442,8 +2385,8 @@
       <c r="B20" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C20" t="s">
-        <v>76</v>
+      <c r="C20" s="2">
+        <v>18</v>
       </c>
       <c r="D20" t="s">
         <v>56</v>
@@ -2456,8 +2399,8 @@
       <c r="B21" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C21" t="s">
-        <v>77</v>
+      <c r="C21" s="2">
+        <v>19</v>
       </c>
       <c r="D21" t="s">
         <v>57</v>
@@ -2474,7 +2417,7 @@
         <v>0</v>
       </c>
       <c r="D22" t="s">
-        <v>79</v>
+        <v>59</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -2488,7 +2431,7 @@
         <v>1</v>
       </c>
       <c r="D23" t="s">
-        <v>81</v>
+        <v>61</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -2502,7 +2445,7 @@
         <v>2</v>
       </c>
       <c r="D24" t="s">
-        <v>83</v>
+        <v>63</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -2516,7 +2459,7 @@
         <v>3</v>
       </c>
       <c r="D25" t="s">
-        <v>85</v>
+        <v>65</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -2530,7 +2473,7 @@
         <v>0</v>
       </c>
       <c r="D26" t="s">
-        <v>86</v>
+        <v>66</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -2544,7 +2487,7 @@
         <v>1</v>
       </c>
       <c r="D27" t="s">
-        <v>87</v>
+        <v>67</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -2558,7 +2501,7 @@
         <v>0</v>
       </c>
       <c r="D28" t="s">
-        <v>88</v>
+        <v>68</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -2572,7 +2515,7 @@
         <v>1</v>
       </c>
       <c r="D29" t="s">
-        <v>89</v>
+        <v>69</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -2586,7 +2529,7 @@
         <v>0</v>
       </c>
       <c r="D30" t="s">
-        <v>90</v>
+        <v>70</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -2600,7 +2543,7 @@
         <v>1</v>
       </c>
       <c r="D31" t="s">
-        <v>91</v>
+        <v>71</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -2614,7 +2557,7 @@
         <v>0</v>
       </c>
       <c r="D32" t="s">
-        <v>92</v>
+        <v>72</v>
       </c>
     </row>
     <row r="33" spans="1:4">
@@ -2628,7 +2571,7 @@
         <v>1</v>
       </c>
       <c r="D33" t="s">
-        <v>94</v>
+        <v>74</v>
       </c>
     </row>
     <row r="34" spans="1:4">
@@ -2642,7 +2585,7 @@
         <v>2</v>
       </c>
       <c r="D34" t="s">
-        <v>95</v>
+        <v>75</v>
       </c>
     </row>
     <row r="35" spans="1:4">
@@ -2656,7 +2599,7 @@
         <v>0</v>
       </c>
       <c r="D35" t="s">
-        <v>96</v>
+        <v>76</v>
       </c>
     </row>
     <row r="36" spans="1:4">
@@ -2670,7 +2613,7 @@
         <v>1</v>
       </c>
       <c r="D36" t="s">
-        <v>81</v>
+        <v>61</v>
       </c>
     </row>
     <row r="37" spans="1:4">
@@ -2684,7 +2627,7 @@
         <v>2</v>
       </c>
       <c r="D37" t="s">
-        <v>98</v>
+        <v>78</v>
       </c>
     </row>
     <row r="38" spans="1:4">
@@ -2698,7 +2641,7 @@
         <v>3</v>
       </c>
       <c r="D38" t="s">
-        <v>79</v>
+        <v>59</v>
       </c>
     </row>
     <row r="39" spans="1:4">
@@ -2712,7 +2655,7 @@
         <v>4</v>
       </c>
       <c r="D39" t="s">
-        <v>100</v>
+        <v>80</v>
       </c>
     </row>
     <row r="40" spans="1:4">
@@ -2726,7 +2669,7 @@
         <v>5</v>
       </c>
       <c r="D40" t="s">
-        <v>102</v>
+        <v>82</v>
       </c>
     </row>
     <row r="41" spans="1:4">
@@ -2740,7 +2683,7 @@
         <v>0</v>
       </c>
       <c r="D41" t="s">
-        <v>92</v>
+        <v>72</v>
       </c>
     </row>
     <row r="42" spans="1:4">
@@ -2754,7 +2697,7 @@
         <v>1</v>
       </c>
       <c r="D42" t="s">
-        <v>95</v>
+        <v>75</v>
       </c>
     </row>
     <row r="43" spans="1:4">
@@ -2768,7 +2711,7 @@
         <v>2</v>
       </c>
       <c r="D43" t="s">
-        <v>103</v>
+        <v>83</v>
       </c>
     </row>
     <row r="44" spans="1:4">
@@ -2782,7 +2725,7 @@
         <v>3</v>
       </c>
       <c r="D44" t="s">
-        <v>104</v>
+        <v>84</v>
       </c>
     </row>
     <row r="45" spans="1:4">
@@ -2796,7 +2739,7 @@
         <v>0</v>
       </c>
       <c r="D45" t="s">
-        <v>105</v>
+        <v>85</v>
       </c>
     </row>
     <row r="46" spans="1:4">
@@ -2810,7 +2753,7 @@
         <v>1</v>
       </c>
       <c r="D46" t="s">
-        <v>106</v>
+        <v>86</v>
       </c>
     </row>
     <row r="47" spans="1:4">
@@ -2824,7 +2767,7 @@
         <v>0</v>
       </c>
       <c r="D47" t="s">
-        <v>107</v>
+        <v>87</v>
       </c>
     </row>
     <row r="48" spans="1:4">
@@ -2838,7 +2781,7 @@
         <v>1</v>
       </c>
       <c r="D48" t="s">
-        <v>108</v>
+        <v>88</v>
       </c>
     </row>
     <row r="49" spans="1:4">
@@ -2852,7 +2795,7 @@
         <v>2</v>
       </c>
       <c r="D49" t="s">
-        <v>109</v>
+        <v>89</v>
       </c>
     </row>
     <row r="50" spans="1:4">
@@ -2866,7 +2809,7 @@
         <v>3</v>
       </c>
       <c r="D50" t="s">
-        <v>110</v>
+        <v>90</v>
       </c>
     </row>
     <row r="51" spans="1:4">
@@ -2880,7 +2823,7 @@
         <v>4</v>
       </c>
       <c r="D51" t="s">
-        <v>111</v>
+        <v>91</v>
       </c>
     </row>
     <row r="52" spans="1:4">
@@ -2894,7 +2837,7 @@
         <v>5</v>
       </c>
       <c r="D52" t="s">
-        <v>112</v>
+        <v>92</v>
       </c>
     </row>
     <row r="53" spans="1:4">
@@ -2908,7 +2851,7 @@
         <v>6</v>
       </c>
       <c r="D53" t="s">
-        <v>113</v>
+        <v>93</v>
       </c>
     </row>
     <row r="54" spans="1:4">
@@ -2922,7 +2865,7 @@
         <v>7</v>
       </c>
       <c r="D54" t="s">
-        <v>114</v>
+        <v>94</v>
       </c>
     </row>
     <row r="55" spans="1:4">
@@ -2936,7 +2879,7 @@
         <v>8</v>
       </c>
       <c r="D55" t="s">
-        <v>115</v>
+        <v>95</v>
       </c>
     </row>
     <row r="56" spans="1:4">
@@ -2950,7 +2893,7 @@
         <v>9</v>
       </c>
       <c r="D56" t="s">
-        <v>116</v>
+        <v>96</v>
       </c>
     </row>
     <row r="57" spans="1:4">
@@ -2964,7 +2907,7 @@
         <v>10</v>
       </c>
       <c r="D57" t="s">
-        <v>117</v>
+        <v>97</v>
       </c>
     </row>
     <row r="58" spans="1:4">
@@ -2978,7 +2921,7 @@
         <v>11</v>
       </c>
       <c r="D58" t="s">
-        <v>118</v>
+        <v>98</v>
       </c>
     </row>
     <row r="59" spans="1:4">
@@ -2992,7 +2935,7 @@
         <v>12</v>
       </c>
       <c r="D59" t="s">
-        <v>119</v>
+        <v>99</v>
       </c>
     </row>
     <row r="60" spans="1:4">
@@ -3006,7 +2949,7 @@
         <v>13</v>
       </c>
       <c r="D60" t="s">
-        <v>120</v>
+        <v>100</v>
       </c>
     </row>
     <row r="61" spans="1:4">
@@ -3020,7 +2963,7 @@
         <v>14</v>
       </c>
       <c r="D61" t="s">
-        <v>121</v>
+        <v>101</v>
       </c>
     </row>
     <row r="62" spans="1:4">
@@ -3034,7 +2977,7 @@
         <v>15</v>
       </c>
       <c r="D62" t="s">
-        <v>122</v>
+        <v>102</v>
       </c>
     </row>
     <row r="63" spans="1:4">
@@ -3048,7 +2991,7 @@
         <v>16</v>
       </c>
       <c r="D63" t="s">
-        <v>123</v>
+        <v>103</v>
       </c>
     </row>
     <row r="64" spans="1:4">
@@ -3062,7 +3005,7 @@
         <v>17</v>
       </c>
       <c r="D64" t="s">
-        <v>124</v>
+        <v>104</v>
       </c>
     </row>
     <row r="65" spans="1:4">
@@ -3076,7 +3019,7 @@
         <v>18</v>
       </c>
       <c r="D65" t="s">
-        <v>125</v>
+        <v>105</v>
       </c>
     </row>
     <row r="66" spans="1:4">
@@ -3090,7 +3033,7 @@
         <v>19</v>
       </c>
       <c r="D66" t="s">
-        <v>126</v>
+        <v>106</v>
       </c>
     </row>
     <row r="67" spans="1:4">
@@ -3104,7 +3047,7 @@
         <v>20</v>
       </c>
       <c r="D67" t="s">
-        <v>127</v>
+        <v>107</v>
       </c>
     </row>
     <row r="68" spans="1:4">
@@ -3118,7 +3061,7 @@
         <v>21</v>
       </c>
       <c r="D68" t="s">
-        <v>128</v>
+        <v>108</v>
       </c>
     </row>
     <row r="69" spans="1:4">
@@ -3132,7 +3075,7 @@
         <v>22</v>
       </c>
       <c r="D69" t="s">
-        <v>129</v>
+        <v>109</v>
       </c>
     </row>
     <row r="70" spans="1:4">
@@ -3146,7 +3089,7 @@
         <v>23</v>
       </c>
       <c r="D70" t="s">
-        <v>130</v>
+        <v>110</v>
       </c>
     </row>
     <row r="71" spans="1:4">
@@ -3160,7 +3103,7 @@
         <v>24</v>
       </c>
       <c r="D71" t="s">
-        <v>131</v>
+        <v>111</v>
       </c>
     </row>
     <row r="72" spans="1:4">
@@ -3174,7 +3117,7 @@
         <v>25</v>
       </c>
       <c r="D72" t="s">
-        <v>132</v>
+        <v>112</v>
       </c>
     </row>
     <row r="73" spans="1:4">
@@ -3188,7 +3131,7 @@
         <v>26</v>
       </c>
       <c r="D73" t="s">
-        <v>133</v>
+        <v>113</v>
       </c>
     </row>
     <row r="74" spans="1:4">
@@ -3202,7 +3145,7 @@
         <v>27</v>
       </c>
       <c r="D74" t="s">
-        <v>134</v>
+        <v>114</v>
       </c>
     </row>
     <row r="75" spans="1:4">
@@ -3216,7 +3159,7 @@
         <v>28</v>
       </c>
       <c r="D75" t="s">
-        <v>135</v>
+        <v>115</v>
       </c>
     </row>
     <row r="76" spans="1:4">
@@ -3230,7 +3173,7 @@
         <v>29</v>
       </c>
       <c r="D76" t="s">
-        <v>136</v>
+        <v>116</v>
       </c>
     </row>
     <row r="77" spans="1:4">
@@ -3244,7 +3187,7 @@
         <v>30</v>
       </c>
       <c r="D77" t="s">
-        <v>137</v>
+        <v>117</v>
       </c>
     </row>
     <row r="78" spans="1:4">
@@ -3258,7 +3201,7 @@
         <v>31</v>
       </c>
       <c r="D78" t="s">
-        <v>138</v>
+        <v>118</v>
       </c>
     </row>
     <row r="79" spans="1:4">
@@ -3272,7 +3215,7 @@
         <v>32</v>
       </c>
       <c r="D79" t="s">
-        <v>139</v>
+        <v>119</v>
       </c>
     </row>
     <row r="80" spans="1:4">
@@ -3286,7 +3229,7 @@
         <v>33</v>
       </c>
       <c r="D80" t="s">
-        <v>140</v>
+        <v>120</v>
       </c>
     </row>
     <row r="81" spans="1:4">
@@ -3300,7 +3243,7 @@
         <v>34</v>
       </c>
       <c r="D81" t="s">
-        <v>141</v>
+        <v>121</v>
       </c>
     </row>
     <row r="82" spans="1:4">
@@ -3314,7 +3257,7 @@
         <v>35</v>
       </c>
       <c r="D82" t="s">
-        <v>142</v>
+        <v>122</v>
       </c>
     </row>
     <row r="83" spans="1:4">
@@ -3328,7 +3271,7 @@
         <v>36</v>
       </c>
       <c r="D83" t="s">
-        <v>143</v>
+        <v>123</v>
       </c>
     </row>
     <row r="84" spans="1:4">
@@ -3342,7 +3285,7 @@
         <v>37</v>
       </c>
       <c r="D84" t="s">
-        <v>144</v>
+        <v>124</v>
       </c>
     </row>
     <row r="85" spans="1:4">
@@ -3356,7 +3299,7 @@
         <v>38</v>
       </c>
       <c r="D85" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
     </row>
     <row r="86" spans="1:4">
@@ -3370,7 +3313,7 @@
         <v>39</v>
       </c>
       <c r="D86" t="s">
-        <v>146</v>
+        <v>126</v>
       </c>
     </row>
     <row r="87" spans="1:4">
@@ -3384,7 +3327,7 @@
         <v>40</v>
       </c>
       <c r="D87" t="s">
-        <v>147</v>
+        <v>127</v>
       </c>
     </row>
     <row r="88" spans="1:4">
@@ -3398,7 +3341,7 @@
         <v>41</v>
       </c>
       <c r="D88" t="s">
-        <v>148</v>
+        <v>128</v>
       </c>
     </row>
     <row r="89" spans="1:4">
@@ -3412,7 +3355,7 @@
         <v>42</v>
       </c>
       <c r="D89" t="s">
-        <v>149</v>
+        <v>129</v>
       </c>
     </row>
     <row r="90" spans="1:4">
@@ -3426,7 +3369,7 @@
         <v>43</v>
       </c>
       <c r="D90" t="s">
-        <v>150</v>
+        <v>130</v>
       </c>
     </row>
     <row r="91" spans="1:4">
@@ -3440,7 +3383,7 @@
         <v>44</v>
       </c>
       <c r="D91" t="s">
-        <v>151</v>
+        <v>131</v>
       </c>
     </row>
     <row r="92" spans="1:4">
@@ -3454,7 +3397,7 @@
         <v>45</v>
       </c>
       <c r="D92" t="s">
-        <v>152</v>
+        <v>132</v>
       </c>
     </row>
     <row r="93" spans="1:4">
@@ -3468,7 +3411,7 @@
         <v>46</v>
       </c>
       <c r="D93" t="s">
-        <v>153</v>
+        <v>133</v>
       </c>
     </row>
     <row r="94" spans="1:4">
@@ -3482,7 +3425,7 @@
         <v>47</v>
       </c>
       <c r="D94" t="s">
-        <v>154</v>
+        <v>134</v>
       </c>
     </row>
     <row r="95" spans="1:4">
@@ -3496,7 +3439,7 @@
         <v>48</v>
       </c>
       <c r="D95" t="s">
-        <v>155</v>
+        <v>135</v>
       </c>
     </row>
     <row r="96" spans="1:4">
@@ -3510,7 +3453,7 @@
         <v>49</v>
       </c>
       <c r="D96" t="s">
-        <v>156</v>
+        <v>136</v>
       </c>
     </row>
     <row r="97" spans="1:4">
@@ -3524,7 +3467,7 @@
         <v>50</v>
       </c>
       <c r="D97" t="s">
-        <v>157</v>
+        <v>137</v>
       </c>
     </row>
     <row r="98" spans="1:4">
@@ -3538,7 +3481,7 @@
         <v>51</v>
       </c>
       <c r="D98" t="s">
-        <v>158</v>
+        <v>138</v>
       </c>
     </row>
     <row r="99" spans="1:4">
@@ -3552,7 +3495,7 @@
         <v>52</v>
       </c>
       <c r="D99" t="s">
-        <v>159</v>
+        <v>139</v>
       </c>
     </row>
     <row r="100" spans="1:4">
@@ -3566,7 +3509,7 @@
         <v>53</v>
       </c>
       <c r="D100" t="s">
-        <v>160</v>
+        <v>140</v>
       </c>
     </row>
     <row r="101" spans="1:4">
@@ -3580,7 +3523,7 @@
         <v>54</v>
       </c>
       <c r="D101" t="s">
-        <v>161</v>
+        <v>141</v>
       </c>
     </row>
     <row r="102" spans="1:4">
@@ -3594,7 +3537,7 @@
         <v>55</v>
       </c>
       <c r="D102" t="s">
-        <v>162</v>
+        <v>142</v>
       </c>
     </row>
     <row r="103" spans="1:4">
@@ -3608,7 +3551,7 @@
         <v>56</v>
       </c>
       <c r="D103" t="s">
-        <v>163</v>
+        <v>143</v>
       </c>
     </row>
     <row r="104" spans="1:4">
@@ -3622,7 +3565,7 @@
         <v>57</v>
       </c>
       <c r="D104" t="s">
-        <v>164</v>
+        <v>144</v>
       </c>
     </row>
     <row r="105" spans="1:4">
@@ -3636,7 +3579,7 @@
         <v>58</v>
       </c>
       <c r="D105" t="s">
-        <v>165</v>
+        <v>145</v>
       </c>
     </row>
     <row r="106" spans="1:4">
@@ -3650,7 +3593,7 @@
         <v>59</v>
       </c>
       <c r="D106" t="s">
-        <v>166</v>
+        <v>146</v>
       </c>
     </row>
     <row r="107" spans="1:4">
@@ -3664,7 +3607,7 @@
         <v>60</v>
       </c>
       <c r="D107" t="s">
-        <v>167</v>
+        <v>147</v>
       </c>
     </row>
     <row r="108" spans="1:4">
@@ -3678,7 +3621,7 @@
         <v>61</v>
       </c>
       <c r="D108" t="s">
-        <v>168</v>
+        <v>148</v>
       </c>
     </row>
     <row r="109" spans="1:4">
@@ -3692,7 +3635,7 @@
         <v>62</v>
       </c>
       <c r="D109" t="s">
-        <v>169</v>
+        <v>149</v>
       </c>
     </row>
     <row r="110" spans="1:4">
@@ -3706,7 +3649,7 @@
         <v>63</v>
       </c>
       <c r="D110" t="s">
-        <v>170</v>
+        <v>150</v>
       </c>
     </row>
     <row r="111" spans="1:4">
@@ -3720,7 +3663,7 @@
         <v>64</v>
       </c>
       <c r="D111" t="s">
-        <v>171</v>
+        <v>151</v>
       </c>
     </row>
     <row r="112" spans="1:4">
@@ -3734,7 +3677,7 @@
         <v>65</v>
       </c>
       <c r="D112" t="s">
-        <v>172</v>
+        <v>152</v>
       </c>
     </row>
     <row r="113" spans="1:4">
@@ -3748,7 +3691,7 @@
         <v>66</v>
       </c>
       <c r="D113" t="s">
-        <v>173</v>
+        <v>153</v>
       </c>
     </row>
     <row r="114" spans="1:4">
@@ -3762,7 +3705,7 @@
         <v>67</v>
       </c>
       <c r="D114" t="s">
-        <v>174</v>
+        <v>154</v>
       </c>
     </row>
     <row r="115" spans="1:4">
@@ -3776,7 +3719,7 @@
         <v>68</v>
       </c>
       <c r="D115" t="s">
-        <v>175</v>
+        <v>155</v>
       </c>
     </row>
     <row r="116" spans="1:4">
@@ -3790,7 +3733,7 @@
         <v>69</v>
       </c>
       <c r="D116" t="s">
-        <v>176</v>
+        <v>156</v>
       </c>
     </row>
     <row r="117" spans="1:4">
@@ -3804,7 +3747,7 @@
         <v>70</v>
       </c>
       <c r="D117" t="s">
-        <v>177</v>
+        <v>157</v>
       </c>
     </row>
     <row r="118" spans="1:4">
@@ -3818,7 +3761,7 @@
         <v>71</v>
       </c>
       <c r="D118" t="s">
-        <v>178</v>
+        <v>158</v>
       </c>
     </row>
     <row r="119" spans="1:4">
@@ -3832,7 +3775,7 @@
         <v>72</v>
       </c>
       <c r="D119" t="s">
-        <v>179</v>
+        <v>159</v>
       </c>
     </row>
     <row r="120" spans="1:4">
@@ -3846,7 +3789,7 @@
         <v>73</v>
       </c>
       <c r="D120" t="s">
-        <v>180</v>
+        <v>160</v>
       </c>
     </row>
     <row r="121" spans="1:4">
@@ -3860,7 +3803,7 @@
         <v>74</v>
       </c>
       <c r="D121" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
     </row>
     <row r="122" spans="1:4">
@@ -3874,7 +3817,7 @@
         <v>75</v>
       </c>
       <c r="D122" t="s">
-        <v>182</v>
+        <v>162</v>
       </c>
     </row>
     <row r="123" spans="1:4">
@@ -3888,7 +3831,7 @@
         <v>76</v>
       </c>
       <c r="D123" t="s">
-        <v>183</v>
+        <v>163</v>
       </c>
     </row>
     <row r="124" spans="1:4">
@@ -3902,7 +3845,7 @@
         <v>77</v>
       </c>
       <c r="D124" t="s">
-        <v>184</v>
+        <v>164</v>
       </c>
     </row>
     <row r="125" spans="1:4">
@@ -3916,7 +3859,7 @@
         <v>78</v>
       </c>
       <c r="D125" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
     </row>
     <row r="126" spans="1:4">
@@ -3930,7 +3873,7 @@
         <v>79</v>
       </c>
       <c r="D126" t="s">
-        <v>186</v>
+        <v>166</v>
       </c>
     </row>
     <row r="127" spans="1:4">
@@ -3944,7 +3887,7 @@
         <v>80</v>
       </c>
       <c r="D127" t="s">
-        <v>187</v>
+        <v>167</v>
       </c>
     </row>
     <row r="128" spans="1:4">
@@ -3958,7 +3901,7 @@
         <v>81</v>
       </c>
       <c r="D128" t="s">
-        <v>188</v>
+        <v>168</v>
       </c>
     </row>
     <row r="129" spans="1:4">
@@ -3972,7 +3915,7 @@
         <v>82</v>
       </c>
       <c r="D129" t="s">
-        <v>189</v>
+        <v>169</v>
       </c>
     </row>
     <row r="130" spans="1:4">
@@ -3986,7 +3929,7 @@
         <v>83</v>
       </c>
       <c r="D130" t="s">
-        <v>190</v>
+        <v>170</v>
       </c>
     </row>
     <row r="131" spans="1:4">
@@ -4000,7 +3943,7 @@
         <v>84</v>
       </c>
       <c r="D131" t="s">
-        <v>191</v>
+        <v>171</v>
       </c>
     </row>
     <row r="132" spans="1:4">
@@ -4014,7 +3957,7 @@
         <v>85</v>
       </c>
       <c r="D132" t="s">
-        <v>192</v>
+        <v>172</v>
       </c>
     </row>
     <row r="133" spans="1:4">
@@ -4028,7 +3971,7 @@
         <v>86</v>
       </c>
       <c r="D133" t="s">
-        <v>193</v>
+        <v>173</v>
       </c>
     </row>
     <row r="134" spans="1:4">
@@ -4042,7 +3985,7 @@
         <v>87</v>
       </c>
       <c r="D134" t="s">
-        <v>194</v>
+        <v>174</v>
       </c>
     </row>
     <row r="135" spans="1:4">
@@ -4056,7 +3999,7 @@
         <v>88</v>
       </c>
       <c r="D135" t="s">
-        <v>195</v>
+        <v>175</v>
       </c>
     </row>
     <row r="136" spans="1:4">
@@ -4070,7 +4013,7 @@
         <v>89</v>
       </c>
       <c r="D136" t="s">
-        <v>196</v>
+        <v>176</v>
       </c>
     </row>
     <row r="137" spans="1:4">
@@ -4084,7 +4027,7 @@
         <v>90</v>
       </c>
       <c r="D137" t="s">
-        <v>197</v>
+        <v>177</v>
       </c>
     </row>
     <row r="138" spans="1:4">
@@ -4098,7 +4041,7 @@
         <v>91</v>
       </c>
       <c r="D138" t="s">
-        <v>198</v>
+        <v>178</v>
       </c>
     </row>
     <row r="139" spans="1:4">
@@ -4112,7 +4055,7 @@
         <v>92</v>
       </c>
       <c r="D139" t="s">
-        <v>199</v>
+        <v>179</v>
       </c>
     </row>
     <row r="140" spans="1:4">
@@ -4126,7 +4069,7 @@
         <v>93</v>
       </c>
       <c r="D140" t="s">
-        <v>200</v>
+        <v>180</v>
       </c>
     </row>
     <row r="141" spans="1:4">
@@ -4140,7 +4083,7 @@
         <v>94</v>
       </c>
       <c r="D141" t="s">
-        <v>201</v>
+        <v>181</v>
       </c>
     </row>
     <row r="142" spans="1:4">
@@ -4154,7 +4097,7 @@
         <v>95</v>
       </c>
       <c r="D142" t="s">
-        <v>202</v>
+        <v>182</v>
       </c>
     </row>
     <row r="143" spans="1:4">
@@ -4168,7 +4111,7 @@
         <v>96</v>
       </c>
       <c r="D143" t="s">
-        <v>203</v>
+        <v>183</v>
       </c>
     </row>
     <row r="144" spans="1:4">
@@ -4182,7 +4125,7 @@
         <v>97</v>
       </c>
       <c r="D144" t="s">
-        <v>204</v>
+        <v>184</v>
       </c>
     </row>
     <row r="145" spans="1:4">
@@ -4196,7 +4139,7 @@
         <v>98</v>
       </c>
       <c r="D145" t="s">
-        <v>205</v>
+        <v>185</v>
       </c>
     </row>
     <row r="146" spans="1:4">
@@ -4210,7 +4153,7 @@
         <v>99</v>
       </c>
       <c r="D146" t="s">
-        <v>206</v>
+        <v>186</v>
       </c>
     </row>
     <row r="147" spans="1:4">
@@ -4224,7 +4167,7 @@
         <v>100</v>
       </c>
       <c r="D147" t="s">
-        <v>207</v>
+        <v>187</v>
       </c>
     </row>
     <row r="148" spans="1:4">
@@ -4238,7 +4181,7 @@
         <v>101</v>
       </c>
       <c r="D148" t="s">
-        <v>208</v>
+        <v>188</v>
       </c>
     </row>
     <row r="149" spans="1:4">
@@ -4252,7 +4195,7 @@
         <v>102</v>
       </c>
       <c r="D149" t="s">
-        <v>209</v>
+        <v>189</v>
       </c>
     </row>
     <row r="150" spans="1:4">
@@ -4266,7 +4209,7 @@
         <v>103</v>
       </c>
       <c r="D150" t="s">
-        <v>210</v>
+        <v>190</v>
       </c>
     </row>
     <row r="151" spans="1:4">
@@ -4280,7 +4223,7 @@
         <v>104</v>
       </c>
       <c r="D151" t="s">
-        <v>211</v>
+        <v>191</v>
       </c>
     </row>
     <row r="152" spans="1:4">
@@ -4294,7 +4237,7 @@
         <v>105</v>
       </c>
       <c r="D152" t="s">
-        <v>212</v>
+        <v>192</v>
       </c>
     </row>
     <row r="153" spans="1:4">
@@ -4308,7 +4251,7 @@
         <v>106</v>
       </c>
       <c r="D153" t="s">
-        <v>213</v>
+        <v>193</v>
       </c>
     </row>
     <row r="154" spans="1:4">
@@ -4322,7 +4265,7 @@
         <v>107</v>
       </c>
       <c r="D154" t="s">
-        <v>214</v>
+        <v>194</v>
       </c>
     </row>
     <row r="155" spans="1:4">
@@ -4336,7 +4279,7 @@
         <v>108</v>
       </c>
       <c r="D155" t="s">
-        <v>215</v>
+        <v>195</v>
       </c>
     </row>
     <row r="156" spans="1:4">
@@ -4350,7 +4293,7 @@
         <v>109</v>
       </c>
       <c r="D156" t="s">
-        <v>216</v>
+        <v>196</v>
       </c>
     </row>
     <row r="157" spans="1:4">
@@ -4364,7 +4307,7 @@
         <v>110</v>
       </c>
       <c r="D157" t="s">
-        <v>217</v>
+        <v>197</v>
       </c>
     </row>
     <row r="158" spans="1:4">
@@ -4378,7 +4321,7 @@
         <v>111</v>
       </c>
       <c r="D158" t="s">
-        <v>218</v>
+        <v>198</v>
       </c>
     </row>
     <row r="159" spans="1:4">
@@ -4392,7 +4335,7 @@
         <v>112</v>
       </c>
       <c r="D159" t="s">
-        <v>219</v>
+        <v>199</v>
       </c>
     </row>
     <row r="160" spans="1:4">
@@ -4406,7 +4349,7 @@
         <v>113</v>
       </c>
       <c r="D160" t="s">
-        <v>220</v>
+        <v>200</v>
       </c>
     </row>
     <row r="161" spans="1:4">
@@ -4420,7 +4363,7 @@
         <v>114</v>
       </c>
       <c r="D161" t="s">
-        <v>221</v>
+        <v>201</v>
       </c>
     </row>
     <row r="162" spans="1:4">
@@ -4434,7 +4377,7 @@
         <v>115</v>
       </c>
       <c r="D162" t="s">
-        <v>222</v>
+        <v>202</v>
       </c>
     </row>
     <row r="163" spans="1:4">
@@ -4448,7 +4391,7 @@
         <v>116</v>
       </c>
       <c r="D163" t="s">
-        <v>223</v>
+        <v>203</v>
       </c>
     </row>
     <row r="164" spans="1:4">
@@ -4462,7 +4405,7 @@
         <v>117</v>
       </c>
       <c r="D164" t="s">
-        <v>224</v>
+        <v>204</v>
       </c>
     </row>
     <row r="165" spans="1:4">
@@ -4476,7 +4419,7 @@
         <v>118</v>
       </c>
       <c r="D165" t="s">
-        <v>225</v>
+        <v>205</v>
       </c>
     </row>
     <row r="166" spans="1:4">
@@ -4490,7 +4433,7 @@
         <v>119</v>
       </c>
       <c r="D166" t="s">
-        <v>226</v>
+        <v>206</v>
       </c>
     </row>
     <row r="167" spans="1:4">
@@ -4504,7 +4447,7 @@
         <v>120</v>
       </c>
       <c r="D167" t="s">
-        <v>227</v>
+        <v>207</v>
       </c>
     </row>
     <row r="168" spans="1:4">
@@ -4518,7 +4461,7 @@
         <v>121</v>
       </c>
       <c r="D168" t="s">
-        <v>228</v>
+        <v>208</v>
       </c>
     </row>
     <row r="169" spans="1:4">
@@ -4532,7 +4475,7 @@
         <v>122</v>
       </c>
       <c r="D169" t="s">
-        <v>229</v>
+        <v>209</v>
       </c>
     </row>
     <row r="170" spans="1:4">
@@ -4546,7 +4489,7 @@
         <v>123</v>
       </c>
       <c r="D170" t="s">
-        <v>230</v>
+        <v>210</v>
       </c>
     </row>
     <row r="171" spans="1:4">
@@ -4560,7 +4503,7 @@
         <v>124</v>
       </c>
       <c r="D171" t="s">
-        <v>231</v>
+        <v>211</v>
       </c>
     </row>
     <row r="172" spans="1:4">
@@ -4574,7 +4517,7 @@
         <v>125</v>
       </c>
       <c r="D172" t="s">
-        <v>232</v>
+        <v>212</v>
       </c>
     </row>
     <row r="173" spans="1:4">
@@ -4588,7 +4531,7 @@
         <v>126</v>
       </c>
       <c r="D173" t="s">
-        <v>233</v>
+        <v>213</v>
       </c>
     </row>
     <row r="174" spans="1:4">
@@ -4602,7 +4545,7 @@
         <v>127</v>
       </c>
       <c r="D174" t="s">
-        <v>234</v>
+        <v>214</v>
       </c>
     </row>
     <row r="175" spans="1:4">
@@ -4616,7 +4559,7 @@
         <v>128</v>
       </c>
       <c r="D175" t="s">
-        <v>235</v>
+        <v>215</v>
       </c>
     </row>
     <row r="176" spans="1:4">
@@ -4630,7 +4573,7 @@
         <v>129</v>
       </c>
       <c r="D176" t="s">
-        <v>236</v>
+        <v>216</v>
       </c>
     </row>
     <row r="177" spans="1:4">
@@ -4644,7 +4587,7 @@
         <v>130</v>
       </c>
       <c r="D177" t="s">
-        <v>237</v>
+        <v>217</v>
       </c>
     </row>
     <row r="178" spans="1:4">
@@ -4658,7 +4601,7 @@
         <v>131</v>
       </c>
       <c r="D178" t="s">
-        <v>238</v>
+        <v>218</v>
       </c>
     </row>
     <row r="179" spans="1:4">
@@ -4672,7 +4615,7 @@
         <v>132</v>
       </c>
       <c r="D179" t="s">
-        <v>239</v>
+        <v>219</v>
       </c>
     </row>
     <row r="180" spans="1:4">
@@ -4686,7 +4629,7 @@
         <v>133</v>
       </c>
       <c r="D180" t="s">
-        <v>240</v>
+        <v>220</v>
       </c>
     </row>
     <row r="181" spans="1:4">
@@ -4700,7 +4643,7 @@
         <v>134</v>
       </c>
       <c r="D181" t="s">
-        <v>241</v>
+        <v>221</v>
       </c>
     </row>
     <row r="182" spans="1:4">
@@ -4714,7 +4657,7 @@
         <v>135</v>
       </c>
       <c r="D182" t="s">
-        <v>242</v>
+        <v>222</v>
       </c>
     </row>
     <row r="183" spans="1:4">
@@ -4728,7 +4671,7 @@
         <v>136</v>
       </c>
       <c r="D183" t="s">
-        <v>243</v>
+        <v>223</v>
       </c>
     </row>
     <row r="184" spans="1:4">
@@ -4742,7 +4685,7 @@
         <v>137</v>
       </c>
       <c r="D184" t="s">
-        <v>244</v>
+        <v>224</v>
       </c>
     </row>
     <row r="185" spans="1:4">
@@ -4756,7 +4699,7 @@
         <v>138</v>
       </c>
       <c r="D185" t="s">
-        <v>245</v>
+        <v>225</v>
       </c>
     </row>
     <row r="186" spans="1:4">
@@ -4770,7 +4713,7 @@
         <v>139</v>
       </c>
       <c r="D186" t="s">
-        <v>246</v>
+        <v>226</v>
       </c>
     </row>
     <row r="187" spans="1:4">
@@ -4784,7 +4727,7 @@
         <v>140</v>
       </c>
       <c r="D187" t="s">
-        <v>247</v>
+        <v>227</v>
       </c>
     </row>
     <row r="188" spans="1:4">
@@ -4798,7 +4741,7 @@
         <v>141</v>
       </c>
       <c r="D188" t="s">
-        <v>248</v>
+        <v>228</v>
       </c>
     </row>
     <row r="189" spans="1:4">
@@ -4812,7 +4755,7 @@
         <v>142</v>
       </c>
       <c r="D189" t="s">
-        <v>249</v>
+        <v>229</v>
       </c>
     </row>
     <row r="190" spans="1:4">
@@ -4826,7 +4769,7 @@
         <v>143</v>
       </c>
       <c r="D190" t="s">
-        <v>250</v>
+        <v>230</v>
       </c>
     </row>
     <row r="191" spans="1:4">
@@ -4840,7 +4783,7 @@
         <v>144</v>
       </c>
       <c r="D191" t="s">
-        <v>251</v>
+        <v>231</v>
       </c>
     </row>
     <row r="192" spans="1:4">
@@ -4854,7 +4797,7 @@
         <v>145</v>
       </c>
       <c r="D192" t="s">
-        <v>252</v>
+        <v>232</v>
       </c>
     </row>
     <row r="193" spans="1:4">
@@ -4868,7 +4811,7 @@
         <v>146</v>
       </c>
       <c r="D193" t="s">
-        <v>253</v>
+        <v>233</v>
       </c>
     </row>
     <row r="194" spans="1:4">
@@ -4882,7 +4825,7 @@
         <v>147</v>
       </c>
       <c r="D194" t="s">
-        <v>254</v>
+        <v>234</v>
       </c>
     </row>
     <row r="195" spans="1:4">
@@ -4896,7 +4839,7 @@
         <v>148</v>
       </c>
       <c r="D195" t="s">
-        <v>255</v>
+        <v>235</v>
       </c>
     </row>
     <row r="196" spans="1:4">
@@ -4910,7 +4853,7 @@
         <v>149</v>
       </c>
       <c r="D196" t="s">
-        <v>256</v>
+        <v>236</v>
       </c>
     </row>
     <row r="197" spans="1:4">
@@ -4924,7 +4867,7 @@
         <v>150</v>
       </c>
       <c r="D197" t="s">
-        <v>257</v>
+        <v>237</v>
       </c>
     </row>
     <row r="198" spans="1:4">
@@ -4938,7 +4881,7 @@
         <v>0</v>
       </c>
       <c r="D198" t="s">
-        <v>258</v>
+        <v>238</v>
       </c>
     </row>
     <row r="199" spans="1:4">
@@ -4952,7 +4895,7 @@
         <v>1</v>
       </c>
       <c r="D199" t="s">
-        <v>259</v>
+        <v>239</v>
       </c>
     </row>
     <row r="200" spans="1:4">
@@ -4966,7 +4909,7 @@
         <v>0</v>
       </c>
       <c r="D200" t="s">
-        <v>260</v>
+        <v>240</v>
       </c>
     </row>
     <row r="201" spans="1:4">
@@ -4980,7 +4923,7 @@
         <v>1</v>
       </c>
       <c r="D201" t="s">
-        <v>261</v>
+        <v>241</v>
       </c>
     </row>
     <row r="202" spans="1:4">
@@ -4994,7 +4937,7 @@
         <v>2</v>
       </c>
       <c r="D202" t="s">
-        <v>262</v>
+        <v>242</v>
       </c>
     </row>
     <row r="203" spans="1:4">
@@ -5008,7 +4951,7 @@
         <v>3</v>
       </c>
       <c r="D203" t="s">
-        <v>263</v>
+        <v>243</v>
       </c>
     </row>
     <row r="204" spans="1:4">
@@ -5022,7 +4965,7 @@
         <v>4</v>
       </c>
       <c r="D204" t="s">
-        <v>264</v>
+        <v>244</v>
       </c>
     </row>
     <row r="205" spans="1:4">
@@ -5036,7 +4979,7 @@
         <v>0</v>
       </c>
       <c r="D205" t="s">
-        <v>265</v>
+        <v>245</v>
       </c>
     </row>
     <row r="206" spans="1:4">
@@ -5050,7 +4993,7 @@
         <v>1</v>
       </c>
       <c r="D206" t="s">
-        <v>266</v>
+        <v>246</v>
       </c>
     </row>
     <row r="207" spans="1:4">
@@ -5064,7 +5007,7 @@
         <v>0</v>
       </c>
       <c r="D207" t="s">
-        <v>267</v>
+        <v>247</v>
       </c>
     </row>
     <row r="208" spans="1:4">
@@ -5078,7 +5021,7 @@
         <v>1</v>
       </c>
       <c r="D208" t="s">
-        <v>268</v>
+        <v>248</v>
       </c>
     </row>
     <row r="209" spans="1:4">
@@ -5092,7 +5035,7 @@
         <v>0</v>
       </c>
       <c r="D209" t="s">
-        <v>269</v>
+        <v>249</v>
       </c>
     </row>
     <row r="210" spans="1:4">
@@ -5106,7 +5049,7 @@
         <v>1</v>
       </c>
       <c r="D210" t="s">
-        <v>270</v>
+        <v>250</v>
       </c>
     </row>
     <row r="211" spans="1:4">
@@ -5120,7 +5063,7 @@
         <v>2</v>
       </c>
       <c r="D211" t="s">
-        <v>271</v>
+        <v>251</v>
       </c>
     </row>
     <row r="212" spans="1:4">
@@ -5134,7 +5077,7 @@
         <v>0</v>
       </c>
       <c r="D212" t="s">
-        <v>272</v>
+        <v>252</v>
       </c>
     </row>
     <row r="213" spans="1:4">
@@ -5148,7 +5091,7 @@
         <v>1</v>
       </c>
       <c r="D213" t="s">
-        <v>273</v>
+        <v>253</v>
       </c>
     </row>
     <row r="214" spans="1:4">
@@ -5162,7 +5105,7 @@
         <v>2</v>
       </c>
       <c r="D214" t="s">
-        <v>274</v>
+        <v>254</v>
       </c>
     </row>
     <row r="215" spans="1:4">
@@ -5176,7 +5119,7 @@
         <v>3</v>
       </c>
       <c r="D215" t="s">
-        <v>275</v>
+        <v>255</v>
       </c>
     </row>
     <row r="216" spans="1:4">
@@ -5190,7 +5133,7 @@
         <v>4</v>
       </c>
       <c r="D216" t="s">
-        <v>276</v>
+        <v>256</v>
       </c>
     </row>
     <row r="217" spans="1:4">
@@ -5204,7 +5147,7 @@
         <v>5</v>
       </c>
       <c r="D217" t="s">
-        <v>277</v>
+        <v>257</v>
       </c>
     </row>
     <row r="218" spans="1:4">
@@ -5218,7 +5161,7 @@
         <v>0</v>
       </c>
       <c r="D218" t="s">
-        <v>92</v>
+        <v>72</v>
       </c>
     </row>
     <row r="219" spans="1:4">
@@ -5232,7 +5175,7 @@
         <v>1</v>
       </c>
       <c r="D219" t="s">
-        <v>95</v>
+        <v>75</v>
       </c>
     </row>
     <row r="220" spans="1:4">
@@ -5246,7 +5189,7 @@
         <v>0</v>
       </c>
       <c r="D220" t="s">
-        <v>278</v>
+        <v>258</v>
       </c>
     </row>
     <row r="221" spans="1:4">
@@ -5260,7 +5203,7 @@
         <v>1</v>
       </c>
       <c r="D221" t="s">
-        <v>279</v>
+        <v>259</v>
       </c>
     </row>
     <row r="222" spans="1:4">
@@ -5274,7 +5217,7 @@
         <v>2</v>
       </c>
       <c r="D222" t="s">
-        <v>280</v>
+        <v>260</v>
       </c>
     </row>
     <row r="223" spans="1:4">
@@ -5288,7 +5231,7 @@
         <v>3</v>
       </c>
       <c r="D223" t="s">
-        <v>281</v>
+        <v>261</v>
       </c>
     </row>
     <row r="224" spans="1:4">
@@ -5302,7 +5245,7 @@
         <v>0</v>
       </c>
       <c r="D224" t="s">
-        <v>282</v>
+        <v>262</v>
       </c>
     </row>
     <row r="225" spans="1:4">
@@ -5316,7 +5259,7 @@
         <v>1</v>
       </c>
       <c r="D225" t="s">
-        <v>283</v>
+        <v>263</v>
       </c>
     </row>
     <row r="226" spans="1:4">
@@ -5330,7 +5273,7 @@
         <v>2</v>
       </c>
       <c r="D226" t="s">
-        <v>284</v>
+        <v>264</v>
       </c>
     </row>
     <row r="227" spans="1:4">
@@ -5344,7 +5287,7 @@
         <v>3</v>
       </c>
       <c r="D227" t="s">
-        <v>285</v>
+        <v>265</v>
       </c>
     </row>
     <row r="228" spans="1:4">
@@ -5358,7 +5301,7 @@
         <v>4</v>
       </c>
       <c r="D228" t="s">
-        <v>286</v>
+        <v>266</v>
       </c>
     </row>
     <row r="229" spans="1:4">
@@ -5372,7 +5315,7 @@
         <v>5</v>
       </c>
       <c r="D229" t="s">
-        <v>287</v>
+        <v>267</v>
       </c>
     </row>
     <row r="230" spans="1:4">
@@ -5386,7 +5329,7 @@
         <v>6</v>
       </c>
       <c r="D230" t="s">
-        <v>288</v>
+        <v>268</v>
       </c>
     </row>
     <row r="231" spans="1:4">
@@ -5400,7 +5343,7 @@
         <v>7</v>
       </c>
       <c r="D231" t="s">
-        <v>289</v>
+        <v>269</v>
       </c>
     </row>
     <row r="232" spans="1:4">
@@ -5414,7 +5357,7 @@
         <v>8</v>
       </c>
       <c r="D232" t="s">
-        <v>290</v>
+        <v>270</v>
       </c>
     </row>
     <row r="233" spans="1:4">
@@ -5428,7 +5371,7 @@
         <v>9</v>
       </c>
       <c r="D233" t="s">
-        <v>291</v>
+        <v>271</v>
       </c>
     </row>
     <row r="234" spans="1:4">
@@ -5442,7 +5385,7 @@
         <v>10</v>
       </c>
       <c r="D234" t="s">
-        <v>292</v>
+        <v>272</v>
       </c>
     </row>
     <row r="235" spans="1:4">
@@ -5456,7 +5399,7 @@
         <v>11</v>
       </c>
       <c r="D235" t="s">
-        <v>293</v>
+        <v>273</v>
       </c>
     </row>
     <row r="236" spans="1:4">
@@ -5470,7 +5413,7 @@
         <v>12</v>
       </c>
       <c r="D236" t="s">
-        <v>294</v>
+        <v>274</v>
       </c>
     </row>
     <row r="237" spans="1:4">
@@ -5484,7 +5427,7 @@
         <v>13</v>
       </c>
       <c r="D237" t="s">
-        <v>295</v>
+        <v>275</v>
       </c>
     </row>
     <row r="238" spans="1:4">
@@ -5498,7 +5441,7 @@
         <v>14</v>
       </c>
       <c r="D238" t="s">
-        <v>296</v>
+        <v>276</v>
       </c>
     </row>
     <row r="239" spans="1:4">
@@ -5512,7 +5455,7 @@
         <v>15</v>
       </c>
       <c r="D239" t="s">
-        <v>297</v>
+        <v>277</v>
       </c>
     </row>
     <row r="240" spans="1:4">
@@ -5526,7 +5469,7 @@
         <v>16</v>
       </c>
       <c r="D240" t="s">
-        <v>298</v>
+        <v>278</v>
       </c>
     </row>
     <row r="241" spans="1:4">
@@ -5540,7 +5483,7 @@
         <v>17</v>
       </c>
       <c r="D241" t="s">
-        <v>299</v>
+        <v>279</v>
       </c>
     </row>
     <row r="242" spans="1:4">
@@ -5554,7 +5497,7 @@
         <v>18</v>
       </c>
       <c r="D242" t="s">
-        <v>300</v>
+        <v>280</v>
       </c>
     </row>
     <row r="243" spans="1:4">
@@ -5568,7 +5511,7 @@
         <v>19</v>
       </c>
       <c r="D243" t="s">
-        <v>301</v>
+        <v>281</v>
       </c>
     </row>
     <row r="244" spans="1:4">
@@ -5582,7 +5525,7 @@
         <v>20</v>
       </c>
       <c r="D244" t="s">
-        <v>302</v>
+        <v>282</v>
       </c>
     </row>
     <row r="245" spans="1:4">
@@ -5596,7 +5539,7 @@
         <v>21</v>
       </c>
       <c r="D245" t="s">
-        <v>303</v>
+        <v>283</v>
       </c>
     </row>
     <row r="246" spans="1:4">
@@ -5610,7 +5553,7 @@
         <v>22</v>
       </c>
       <c r="D246" t="s">
-        <v>304</v>
+        <v>284</v>
       </c>
     </row>
     <row r="247" spans="1:4">
@@ -5624,7 +5567,7 @@
         <v>23</v>
       </c>
       <c r="D247" t="s">
-        <v>305</v>
+        <v>285</v>
       </c>
     </row>
     <row r="248" spans="1:4">
@@ -5638,7 +5581,7 @@
         <v>24</v>
       </c>
       <c r="D248" t="s">
-        <v>306</v>
+        <v>286</v>
       </c>
     </row>
     <row r="249" spans="1:4">
@@ -5652,7 +5595,7 @@
         <v>25</v>
       </c>
       <c r="D249" t="s">
-        <v>307</v>
+        <v>287</v>
       </c>
     </row>
     <row r="250" spans="1:4">
@@ -5666,7 +5609,7 @@
         <v>26</v>
       </c>
       <c r="D250" t="s">
-        <v>308</v>
+        <v>288</v>
       </c>
     </row>
     <row r="251" spans="1:4">
@@ -5680,7 +5623,7 @@
         <v>27</v>
       </c>
       <c r="D251" t="s">
-        <v>309</v>
+        <v>289</v>
       </c>
     </row>
     <row r="252" spans="1:4">
@@ -5694,7 +5637,7 @@
         <v>28</v>
       </c>
       <c r="D252" t="s">
-        <v>310</v>
+        <v>290</v>
       </c>
     </row>
     <row r="253" spans="1:4">
@@ -5708,7 +5651,7 @@
         <v>29</v>
       </c>
       <c r="D253" t="s">
-        <v>311</v>
+        <v>291</v>
       </c>
     </row>
     <row r="254" spans="1:4">
@@ -5722,7 +5665,7 @@
         <v>30</v>
       </c>
       <c r="D254" t="s">
-        <v>312</v>
+        <v>292</v>
       </c>
     </row>
     <row r="255" spans="1:4">
@@ -5736,7 +5679,7 @@
         <v>31</v>
       </c>
       <c r="D255" t="s">
-        <v>313</v>
+        <v>293</v>
       </c>
     </row>
     <row r="256" spans="1:4">
@@ -5750,7 +5693,7 @@
         <v>32</v>
       </c>
       <c r="D256" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
     </row>
     <row r="257" spans="1:4">
@@ -5764,7 +5707,7 @@
         <v>33</v>
       </c>
       <c r="D257" t="s">
-        <v>314</v>
+        <v>294</v>
       </c>
     </row>
     <row r="258" spans="1:4">
@@ -5778,7 +5721,7 @@
         <v>34</v>
       </c>
       <c r="D258" t="s">
-        <v>315</v>
+        <v>295</v>
       </c>
     </row>
     <row r="259" spans="1:4">
@@ -5792,7 +5735,7 @@
         <v>35</v>
       </c>
       <c r="D259" t="s">
-        <v>316</v>
+        <v>296</v>
       </c>
     </row>
     <row r="260" spans="1:4">
@@ -5806,7 +5749,7 @@
         <v>36</v>
       </c>
       <c r="D260" t="s">
-        <v>317</v>
+        <v>297</v>
       </c>
     </row>
     <row r="261" spans="1:4">
@@ -5820,7 +5763,7 @@
         <v>37</v>
       </c>
       <c r="D261" t="s">
-        <v>318</v>
+        <v>298</v>
       </c>
     </row>
     <row r="262" spans="1:4">
@@ -5834,7 +5777,7 @@
         <v>38</v>
       </c>
       <c r="D262" t="s">
-        <v>319</v>
+        <v>299</v>
       </c>
     </row>
     <row r="263" spans="1:4">
@@ -5848,7 +5791,7 @@
         <v>39</v>
       </c>
       <c r="D263" t="s">
-        <v>320</v>
+        <v>300</v>
       </c>
     </row>
     <row r="264" spans="1:4">
@@ -5862,7 +5805,7 @@
         <v>40</v>
       </c>
       <c r="D264" t="s">
-        <v>321</v>
+        <v>301</v>
       </c>
     </row>
     <row r="265" spans="1:4">
@@ -5876,7 +5819,7 @@
         <v>41</v>
       </c>
       <c r="D265" t="s">
-        <v>322</v>
+        <v>302</v>
       </c>
     </row>
     <row r="266" spans="1:4">
@@ -5890,7 +5833,7 @@
         <v>42</v>
       </c>
       <c r="D266" t="s">
-        <v>323</v>
+        <v>303</v>
       </c>
     </row>
     <row r="267" spans="1:4">
@@ -5904,7 +5847,7 @@
         <v>43</v>
       </c>
       <c r="D267" t="s">
-        <v>324</v>
+        <v>304</v>
       </c>
     </row>
     <row r="268" spans="1:4">
@@ -5918,7 +5861,7 @@
         <v>44</v>
       </c>
       <c r="D268" t="s">
-        <v>325</v>
+        <v>305</v>
       </c>
     </row>
     <row r="269" spans="1:4">
@@ -5932,7 +5875,7 @@
         <v>45</v>
       </c>
       <c r="D269" t="s">
-        <v>326</v>
+        <v>306</v>
       </c>
     </row>
     <row r="270" spans="1:4">
@@ -5946,7 +5889,7 @@
         <v>46</v>
       </c>
       <c r="D270" t="s">
-        <v>327</v>
+        <v>307</v>
       </c>
     </row>
     <row r="271" spans="1:4">
@@ -5960,7 +5903,7 @@
         <v>47</v>
       </c>
       <c r="D271" t="s">
-        <v>328</v>
+        <v>308</v>
       </c>
     </row>
     <row r="272" spans="1:4">
@@ -5974,7 +5917,7 @@
         <v>48</v>
       </c>
       <c r="D272" t="s">
-        <v>329</v>
+        <v>309</v>
       </c>
     </row>
     <row r="273" spans="1:4">
@@ -5988,7 +5931,7 @@
         <v>49</v>
       </c>
       <c r="D273" t="s">
-        <v>330</v>
+        <v>310</v>
       </c>
     </row>
     <row r="274" spans="1:4">
@@ -6002,7 +5945,7 @@
         <v>50</v>
       </c>
       <c r="D274" t="s">
-        <v>331</v>
+        <v>311</v>
       </c>
     </row>
     <row r="275" spans="1:4">
@@ -6016,7 +5959,7 @@
         <v>51</v>
       </c>
       <c r="D275" t="s">
-        <v>332</v>
+        <v>312</v>
       </c>
     </row>
     <row r="276" spans="1:4">
@@ -6030,7 +5973,7 @@
         <v>52</v>
       </c>
       <c r="D276" t="s">
-        <v>333</v>
+        <v>313</v>
       </c>
     </row>
     <row r="277" spans="1:4">
@@ -6044,7 +5987,7 @@
         <v>53</v>
       </c>
       <c r="D277" t="s">
-        <v>334</v>
+        <v>314</v>
       </c>
     </row>
     <row r="278" spans="1:4">
@@ -6058,7 +6001,7 @@
         <v>54</v>
       </c>
       <c r="D278" t="s">
-        <v>335</v>
+        <v>315</v>
       </c>
     </row>
     <row r="279" spans="1:4">
@@ -6072,7 +6015,7 @@
         <v>55</v>
       </c>
       <c r="D279" t="s">
-        <v>336</v>
+        <v>316</v>
       </c>
     </row>
     <row r="280" spans="1:4">
@@ -6086,7 +6029,7 @@
         <v>56</v>
       </c>
       <c r="D280" t="s">
-        <v>337</v>
+        <v>317</v>
       </c>
     </row>
     <row r="281" spans="1:4">
@@ -6100,7 +6043,7 @@
         <v>57</v>
       </c>
       <c r="D281" t="s">
-        <v>338</v>
+        <v>318</v>
       </c>
     </row>
     <row r="282" spans="1:4">
@@ -6114,7 +6057,7 @@
         <v>58</v>
       </c>
       <c r="D282" t="s">
-        <v>339</v>
+        <v>319</v>
       </c>
     </row>
     <row r="283" spans="1:4">
@@ -6128,7 +6071,7 @@
         <v>59</v>
       </c>
       <c r="D283" t="s">
-        <v>340</v>
+        <v>320</v>
       </c>
     </row>
     <row r="284" spans="1:4">
@@ -6142,7 +6085,7 @@
         <v>60</v>
       </c>
       <c r="D284" t="s">
-        <v>341</v>
+        <v>321</v>
       </c>
     </row>
     <row r="285" spans="1:4">
@@ -6156,7 +6099,7 @@
         <v>61</v>
       </c>
       <c r="D285" t="s">
-        <v>342</v>
+        <v>322</v>
       </c>
     </row>
     <row r="286" spans="1:4">
@@ -6170,7 +6113,7 @@
         <v>62</v>
       </c>
       <c r="D286" t="s">
-        <v>343</v>
+        <v>323</v>
       </c>
     </row>
     <row r="287" spans="1:4">
@@ -6184,7 +6127,7 @@
         <v>63</v>
       </c>
       <c r="D287" t="s">
-        <v>344</v>
+        <v>324</v>
       </c>
     </row>
     <row r="288" spans="1:4">
@@ -6198,7 +6141,7 @@
         <v>64</v>
       </c>
       <c r="D288" t="s">
-        <v>345</v>
+        <v>325</v>
       </c>
     </row>
     <row r="289" spans="1:4">
@@ -6212,7 +6155,7 @@
         <v>65</v>
       </c>
       <c r="D289" t="s">
-        <v>346</v>
+        <v>326</v>
       </c>
     </row>
     <row r="290" spans="1:4">
@@ -6226,7 +6169,7 @@
         <v>66</v>
       </c>
       <c r="D290" t="s">
-        <v>347</v>
+        <v>327</v>
       </c>
     </row>
     <row r="291" spans="1:4">
@@ -6240,7 +6183,7 @@
         <v>67</v>
       </c>
       <c r="D291" t="s">
-        <v>348</v>
+        <v>328</v>
       </c>
     </row>
     <row r="292" spans="1:4">
@@ -6254,7 +6197,7 @@
         <v>68</v>
       </c>
       <c r="D292" t="s">
-        <v>349</v>
+        <v>329</v>
       </c>
     </row>
     <row r="293" spans="1:4">
@@ -6268,7 +6211,7 @@
         <v>69</v>
       </c>
       <c r="D293" t="s">
-        <v>350</v>
+        <v>330</v>
       </c>
     </row>
     <row r="294" spans="1:4">
@@ -6282,7 +6225,7 @@
         <v>70</v>
       </c>
       <c r="D294" t="s">
-        <v>351</v>
+        <v>331</v>
       </c>
     </row>
     <row r="295" spans="1:4">
@@ -6296,7 +6239,7 @@
         <v>71</v>
       </c>
       <c r="D295" t="s">
-        <v>352</v>
+        <v>332</v>
       </c>
     </row>
     <row r="296" spans="1:4">
@@ -6310,7 +6253,7 @@
         <v>72</v>
       </c>
       <c r="D296" t="s">
-        <v>353</v>
+        <v>333</v>
       </c>
     </row>
     <row r="297" spans="1:4">
@@ -6324,7 +6267,7 @@
         <v>73</v>
       </c>
       <c r="D297" t="s">
-        <v>354</v>
+        <v>334</v>
       </c>
     </row>
     <row r="298" spans="1:4">
@@ -6338,7 +6281,7 @@
         <v>74</v>
       </c>
       <c r="D298" t="s">
-        <v>355</v>
+        <v>335</v>
       </c>
     </row>
     <row r="299" spans="1:4">
@@ -6352,7 +6295,7 @@
         <v>75</v>
       </c>
       <c r="D299" t="s">
-        <v>356</v>
+        <v>336</v>
       </c>
     </row>
     <row r="300" spans="1:4">
@@ -6366,7 +6309,7 @@
         <v>76</v>
       </c>
       <c r="D300" t="s">
-        <v>357</v>
+        <v>337</v>
       </c>
     </row>
     <row r="301" spans="1:4">
@@ -6380,7 +6323,7 @@
         <v>0</v>
       </c>
       <c r="D301" t="s">
-        <v>105</v>
+        <v>85</v>
       </c>
     </row>
     <row r="302" spans="1:4">
@@ -6394,7 +6337,7 @@
         <v>1</v>
       </c>
       <c r="D302" t="s">
-        <v>106</v>
+        <v>86</v>
       </c>
     </row>
     <row r="303" spans="1:4">
@@ -6408,7 +6351,7 @@
         <v>0</v>
       </c>
       <c r="D303" t="s">
-        <v>358</v>
+        <v>338</v>
       </c>
     </row>
     <row r="304" spans="1:4">
@@ -6422,7 +6365,7 @@
         <v>1</v>
       </c>
       <c r="D304" t="s">
-        <v>359</v>
+        <v>339</v>
       </c>
     </row>
     <row r="305" spans="1:4">
@@ -6436,7 +6379,7 @@
         <v>0</v>
       </c>
       <c r="D305" t="s">
-        <v>360</v>
+        <v>340</v>
       </c>
     </row>
     <row r="306" spans="1:4">
@@ -6450,7 +6393,7 @@
         <v>1</v>
       </c>
       <c r="D306" t="s">
-        <v>361</v>
+        <v>341</v>
       </c>
     </row>
     <row r="307" spans="1:4">
@@ -6464,7 +6407,7 @@
         <v>2</v>
       </c>
       <c r="D307" t="s">
-        <v>362</v>
+        <v>342</v>
       </c>
     </row>
     <row r="308" spans="1:4">
@@ -6478,7 +6421,7 @@
         <v>0</v>
       </c>
       <c r="D308" t="s">
-        <v>363</v>
+        <v>343</v>
       </c>
     </row>
     <row r="309" spans="1:4">
@@ -6492,7 +6435,7 @@
         <v>1</v>
       </c>
       <c r="D309" t="s">
-        <v>364</v>
+        <v>344</v>
       </c>
     </row>
     <row r="310" spans="1:4">
@@ -6506,7 +6449,7 @@
         <v>0</v>
       </c>
       <c r="D310" t="s">
-        <v>374</v>
+        <v>354</v>
       </c>
     </row>
     <row r="311" spans="1:4">
@@ -6520,7 +6463,7 @@
         <v>1</v>
       </c>
       <c r="D311" t="s">
-        <v>370</v>
+        <v>350</v>
       </c>
     </row>
     <row r="312" spans="1:4">
@@ -6534,7 +6477,7 @@
         <v>2</v>
       </c>
       <c r="D312" t="s">
-        <v>367</v>
+        <v>347</v>
       </c>
     </row>
     <row r="313" spans="1:4">
@@ -6548,7 +6491,7 @@
         <v>3</v>
       </c>
       <c r="D313" t="s">
-        <v>369</v>
+        <v>349</v>
       </c>
     </row>
     <row r="314" spans="1:4">
@@ -6562,7 +6505,7 @@
         <v>4</v>
       </c>
       <c r="D314" t="s">
-        <v>366</v>
+        <v>346</v>
       </c>
     </row>
     <row r="315" spans="1:4">
@@ -6576,7 +6519,7 @@
         <v>5</v>
       </c>
       <c r="D315" t="s">
-        <v>373</v>
+        <v>353</v>
       </c>
     </row>
     <row r="316" spans="1:4">
@@ -6590,7 +6533,7 @@
         <v>6</v>
       </c>
       <c r="D316" t="s">
-        <v>372</v>
+        <v>352</v>
       </c>
     </row>
     <row r="317" spans="1:4">
@@ -6604,7 +6547,7 @@
         <v>7</v>
       </c>
       <c r="D317" t="s">
-        <v>365</v>
+        <v>345</v>
       </c>
     </row>
     <row r="318" spans="1:4">
@@ -6618,7 +6561,7 @@
         <v>8</v>
       </c>
       <c r="D318" t="s">
-        <v>368</v>
+        <v>348</v>
       </c>
     </row>
     <row r="319" spans="1:4">
@@ -6632,7 +6575,7 @@
         <v>9</v>
       </c>
       <c r="D319" t="s">
-        <v>371</v>
+        <v>351</v>
       </c>
     </row>
     <row r="320" spans="1:4">
@@ -6646,7 +6589,7 @@
         <v>0</v>
       </c>
       <c r="D320" t="s">
-        <v>92</v>
+        <v>72</v>
       </c>
     </row>
     <row r="321" spans="1:4">
@@ -6660,7 +6603,7 @@
         <v>1</v>
       </c>
       <c r="D321" t="s">
-        <v>94</v>
+        <v>74</v>
       </c>
     </row>
     <row r="322" spans="1:4">
@@ -6674,7 +6617,7 @@
         <v>2</v>
       </c>
       <c r="D322" t="s">
-        <v>95</v>
+        <v>75</v>
       </c>
     </row>
     <row r="323" spans="1:4">
@@ -6688,7 +6631,7 @@
         <v>0</v>
       </c>
       <c r="D323" t="s">
-        <v>87</v>
+        <v>67</v>
       </c>
     </row>
     <row r="324" spans="1:4">
@@ -6702,7 +6645,7 @@
         <v>1</v>
       </c>
       <c r="D324" t="s">
-        <v>375</v>
+        <v>355</v>
       </c>
     </row>
     <row r="325" spans="1:4">
@@ -6716,7 +6659,7 @@
         <v>2</v>
       </c>
       <c r="D325" t="s">
-        <v>376</v>
+        <v>356</v>
       </c>
     </row>
     <row r="326" spans="1:4">
@@ -6730,7 +6673,7 @@
         <v>3</v>
       </c>
       <c r="D326" t="s">
-        <v>376</v>
+        <v>356</v>
       </c>
     </row>
     <row r="327" spans="1:4">
@@ -6744,7 +6687,7 @@
         <v>0</v>
       </c>
       <c r="D327" t="s">
-        <v>377</v>
+        <v>357</v>
       </c>
     </row>
     <row r="328" spans="1:4">
@@ -6758,7 +6701,7 @@
         <v>1</v>
       </c>
       <c r="D328" t="s">
-        <v>378</v>
+        <v>358</v>
       </c>
     </row>
     <row r="329" spans="1:4">
@@ -6772,7 +6715,7 @@
         <v>2</v>
       </c>
       <c r="D329" t="s">
-        <v>379</v>
+        <v>359</v>
       </c>
     </row>
     <row r="330" spans="1:4">
@@ -6786,7 +6729,7 @@
         <v>0</v>
       </c>
       <c r="D330" t="s">
-        <v>380</v>
+        <v>360</v>
       </c>
     </row>
     <row r="331" spans="1:4">
@@ -6800,7 +6743,7 @@
         <v>1</v>
       </c>
       <c r="D331" t="s">
-        <v>381</v>
+        <v>361</v>
       </c>
     </row>
     <row r="332" spans="1:4">
@@ -6814,7 +6757,7 @@
         <v>2</v>
       </c>
       <c r="D332" t="s">
-        <v>382</v>
+        <v>362</v>
       </c>
     </row>
     <row r="333" spans="1:4">
@@ -6828,7 +6771,7 @@
         <v>3</v>
       </c>
       <c r="D333" t="s">
-        <v>383</v>
+        <v>363</v>
       </c>
     </row>
     <row r="334" spans="1:4">
@@ -6842,7 +6785,7 @@
         <v>4</v>
       </c>
       <c r="D334" t="s">
-        <v>384</v>
+        <v>364</v>
       </c>
     </row>
     <row r="335" spans="1:4">
@@ -6856,7 +6799,7 @@
         <v>0</v>
       </c>
       <c r="D335" t="s">
-        <v>385</v>
+        <v>365</v>
       </c>
     </row>
     <row r="336" spans="1:4">
@@ -6870,7 +6813,7 @@
         <v>1</v>
       </c>
       <c r="D336" t="s">
-        <v>386</v>
+        <v>366</v>
       </c>
     </row>
     <row r="337" spans="1:4">
@@ -6884,7 +6827,7 @@
         <v>2</v>
       </c>
       <c r="D337" t="s">
-        <v>78</v>
+        <v>58</v>
       </c>
     </row>
     <row r="338" spans="1:4">
@@ -6898,7 +6841,7 @@
         <v>3</v>
       </c>
       <c r="D338" t="s">
-        <v>387</v>
+        <v>367</v>
       </c>
     </row>
     <row r="339" spans="1:4">
@@ -6912,7 +6855,7 @@
         <v>4</v>
       </c>
       <c r="D339" t="s">
-        <v>388</v>
+        <v>368</v>
       </c>
     </row>
     <row r="340" spans="1:4">
@@ -6926,7 +6869,7 @@
         <v>5</v>
       </c>
       <c r="D340" t="s">
-        <v>389</v>
+        <v>369</v>
       </c>
     </row>
     <row r="341" spans="1:4">
@@ -6940,7 +6883,7 @@
         <v>6</v>
       </c>
       <c r="D341" t="s">
-        <v>390</v>
+        <v>370</v>
       </c>
     </row>
     <row r="342" spans="1:4">
@@ -6954,7 +6897,7 @@
         <v>7</v>
       </c>
       <c r="D342" t="s">
-        <v>391</v>
+        <v>371</v>
       </c>
     </row>
     <row r="343" spans="1:4">
@@ -6968,7 +6911,7 @@
         <v>8</v>
       </c>
       <c r="D343" t="s">
-        <v>392</v>
+        <v>372</v>
       </c>
     </row>
     <row r="344" spans="1:4">
@@ -6982,7 +6925,7 @@
         <v>9</v>
       </c>
       <c r="D344" t="s">
-        <v>393</v>
+        <v>373</v>
       </c>
     </row>
     <row r="345" spans="1:4">
@@ -6996,7 +6939,7 @@
         <v>10</v>
       </c>
       <c r="D345" t="s">
-        <v>394</v>
+        <v>374</v>
       </c>
     </row>
     <row r="346" spans="1:4">
@@ -7010,7 +6953,7 @@
         <v>11</v>
       </c>
       <c r="D346" t="s">
-        <v>395</v>
+        <v>375</v>
       </c>
     </row>
     <row r="347" spans="1:4">
@@ -7024,7 +6967,7 @@
         <v>12</v>
       </c>
       <c r="D347" t="s">
-        <v>396</v>
+        <v>376</v>
       </c>
     </row>
     <row r="348" spans="1:4">
@@ -7038,7 +6981,7 @@
         <v>13</v>
       </c>
       <c r="D348" t="s">
-        <v>397</v>
+        <v>377</v>
       </c>
     </row>
     <row r="349" spans="1:4">
@@ -7052,7 +6995,7 @@
         <v>14</v>
       </c>
       <c r="D349" t="s">
-        <v>99</v>
+        <v>79</v>
       </c>
     </row>
     <row r="350" spans="1:4">
@@ -7066,7 +7009,7 @@
         <v>15</v>
       </c>
       <c r="D350" t="s">
-        <v>398</v>
+        <v>378</v>
       </c>
     </row>
     <row r="351" spans="1:4">
@@ -7080,7 +7023,7 @@
         <v>16</v>
       </c>
       <c r="D351" t="s">
-        <v>399</v>
+        <v>379</v>
       </c>
     </row>
     <row r="352" spans="1:4">
@@ -7094,7 +7037,7 @@
         <v>17</v>
       </c>
       <c r="D352" t="s">
-        <v>80</v>
+        <v>60</v>
       </c>
     </row>
     <row r="353" spans="1:4">
@@ -7108,7 +7051,7 @@
         <v>18</v>
       </c>
       <c r="D353" t="s">
-        <v>97</v>
+        <v>77</v>
       </c>
     </row>
     <row r="354" spans="1:4">
@@ -7122,7 +7065,7 @@
         <v>19</v>
       </c>
       <c r="D354" t="s">
-        <v>400</v>
+        <v>380</v>
       </c>
     </row>
     <row r="355" spans="1:4">
@@ -7136,7 +7079,7 @@
         <v>20</v>
       </c>
       <c r="D355" t="s">
-        <v>82</v>
+        <v>62</v>
       </c>
     </row>
     <row r="356" spans="1:4">
@@ -7150,7 +7093,7 @@
         <v>21</v>
       </c>
       <c r="D356" t="s">
-        <v>401</v>
+        <v>381</v>
       </c>
     </row>
     <row r="357" spans="1:4">
@@ -7164,7 +7107,7 @@
         <v>22</v>
       </c>
       <c r="D357" t="s">
-        <v>402</v>
+        <v>382</v>
       </c>
     </row>
     <row r="358" spans="1:4">
@@ -7178,7 +7121,7 @@
         <v>23</v>
       </c>
       <c r="D358" t="s">
-        <v>403</v>
+        <v>383</v>
       </c>
     </row>
     <row r="359" spans="1:4">
@@ -7192,7 +7135,7 @@
         <v>24</v>
       </c>
       <c r="D359" t="s">
-        <v>404</v>
+        <v>384</v>
       </c>
     </row>
     <row r="360" spans="1:4">
@@ -7206,7 +7149,7 @@
         <v>25</v>
       </c>
       <c r="D360" t="s">
-        <v>84</v>
+        <v>64</v>
       </c>
     </row>
     <row r="361" spans="1:4">
@@ -7220,7 +7163,7 @@
         <v>26</v>
       </c>
       <c r="D361" t="s">
-        <v>101</v>
+        <v>81</v>
       </c>
     </row>
     <row r="362" spans="1:4">
@@ -7234,7 +7177,7 @@
         <v>27</v>
       </c>
       <c r="D362" t="s">
-        <v>93</v>
+        <v>73</v>
       </c>
     </row>
     <row r="363" spans="1:4">
@@ -7248,7 +7191,7 @@
         <v>1</v>
       </c>
       <c r="D363" t="s">
-        <v>405</v>
+        <v>385</v>
       </c>
     </row>
     <row r="364" spans="1:4">
@@ -7262,7 +7205,7 @@
         <v>2</v>
       </c>
       <c r="D364" t="s">
-        <v>407</v>
+        <v>387</v>
       </c>
     </row>
     <row r="365" spans="1:4">
@@ -7276,7 +7219,7 @@
         <v>3</v>
       </c>
       <c r="D365" t="s">
-        <v>408</v>
+        <v>388</v>
       </c>
     </row>
     <row r="366" spans="1:4">
@@ -7290,7 +7233,7 @@
         <v>4</v>
       </c>
       <c r="D366" t="s">
-        <v>409</v>
+        <v>389</v>
       </c>
     </row>
     <row r="367" spans="1:4">
@@ -7304,7 +7247,7 @@
         <v>0</v>
       </c>
       <c r="D367" t="s">
-        <v>364</v>
+        <v>344</v>
       </c>
     </row>
     <row r="368" spans="1:4">
@@ -7318,7 +7261,7 @@
         <v>1</v>
       </c>
       <c r="D368" t="s">
-        <v>363</v>
+        <v>343</v>
       </c>
     </row>
     <row r="369" spans="1:4">
@@ -7332,7 +7275,7 @@
         <v>0</v>
       </c>
       <c r="D369" t="s">
-        <v>92</v>
+        <v>72</v>
       </c>
     </row>
     <row r="370" spans="1:4">
@@ -7346,7 +7289,7 @@
         <v>1</v>
       </c>
       <c r="D370" t="s">
-        <v>95</v>
+        <v>75</v>
       </c>
     </row>
     <row r="371" spans="1:4">
@@ -7360,7 +7303,7 @@
         <v>0</v>
       </c>
       <c r="D371" t="s">
-        <v>410</v>
+        <v>390</v>
       </c>
     </row>
     <row r="372" spans="1:4">
@@ -7374,7 +7317,7 @@
         <v>1</v>
       </c>
       <c r="D372" t="s">
-        <v>411</v>
+        <v>391</v>
       </c>
     </row>
     <row r="373" spans="1:4">
@@ -7388,7 +7331,7 @@
         <v>2</v>
       </c>
       <c r="D373" t="s">
-        <v>412</v>
+        <v>392</v>
       </c>
     </row>
     <row r="374" spans="1:4">
@@ -7402,7 +7345,7 @@
         <v>3</v>
       </c>
       <c r="D374" t="s">
-        <v>413</v>
+        <v>393</v>
       </c>
     </row>
     <row r="375" spans="1:4">
@@ -7416,7 +7359,7 @@
         <v>4</v>
       </c>
       <c r="D375" t="s">
-        <v>414</v>
+        <v>394</v>
       </c>
     </row>
     <row r="376" spans="1:4">
@@ -7430,7 +7373,7 @@
         <v>5</v>
       </c>
       <c r="D376" t="s">
-        <v>415</v>
+        <v>395</v>
       </c>
     </row>
     <row r="377" spans="1:4">
@@ -7444,7 +7387,7 @@
         <v>6</v>
       </c>
       <c r="D377" t="s">
-        <v>416</v>
+        <v>396</v>
       </c>
     </row>
     <row r="378" spans="1:4">
@@ -7458,7 +7401,7 @@
         <v>7</v>
       </c>
       <c r="D378" t="s">
-        <v>417</v>
+        <v>397</v>
       </c>
     </row>
     <row r="379" spans="1:4">
@@ -7472,7 +7415,7 @@
         <v>8</v>
       </c>
       <c r="D379" t="s">
-        <v>418</v>
+        <v>398</v>
       </c>
     </row>
     <row r="380" spans="1:4">
@@ -7486,7 +7429,7 @@
         <v>9</v>
       </c>
       <c r="D380" t="s">
-        <v>419</v>
+        <v>399</v>
       </c>
     </row>
     <row r="381" spans="1:4">
@@ -7500,7 +7443,7 @@
         <v>10</v>
       </c>
       <c r="D381" t="s">
-        <v>420</v>
+        <v>400</v>
       </c>
     </row>
     <row r="382" spans="1:4">
@@ -7514,7 +7457,7 @@
         <v>11</v>
       </c>
       <c r="D382" t="s">
-        <v>421</v>
+        <v>401</v>
       </c>
     </row>
     <row r="383" spans="1:4">
@@ -7528,7 +7471,7 @@
         <v>12</v>
       </c>
       <c r="D383" t="s">
-        <v>422</v>
+        <v>402</v>
       </c>
     </row>
     <row r="384" spans="1:4">
@@ -7542,7 +7485,7 @@
         <v>13</v>
       </c>
       <c r="D384" t="s">
-        <v>423</v>
+        <v>403</v>
       </c>
     </row>
     <row r="385" spans="1:4">
@@ -7556,7 +7499,7 @@
         <v>0</v>
       </c>
       <c r="D385" t="s">
-        <v>424</v>
+        <v>404</v>
       </c>
     </row>
     <row r="386" spans="1:4">
@@ -7570,7 +7513,7 @@
         <v>1</v>
       </c>
       <c r="D386" t="s">
-        <v>538</v>
+        <v>518</v>
       </c>
     </row>
     <row r="387" spans="1:4">
@@ -7584,7 +7527,7 @@
         <v>2</v>
       </c>
       <c r="D387" t="s">
-        <v>539</v>
+        <v>519</v>
       </c>
     </row>
     <row r="388" spans="1:4">
@@ -7598,7 +7541,7 @@
         <v>3</v>
       </c>
       <c r="D388" t="s">
-        <v>540</v>
+        <v>520</v>
       </c>
     </row>
     <row r="389" spans="1:4">
@@ -7612,7 +7555,7 @@
         <v>4</v>
       </c>
       <c r="D389" t="s">
-        <v>541</v>
+        <v>521</v>
       </c>
     </row>
     <row r="390" spans="1:4">
@@ -7626,7 +7569,7 @@
         <v>5</v>
       </c>
       <c r="D390" t="s">
-        <v>406</v>
+        <v>386</v>
       </c>
     </row>
     <row r="391" spans="1:4">
@@ -7640,7 +7583,7 @@
         <v>6</v>
       </c>
       <c r="D391" t="s">
-        <v>542</v>
+        <v>522</v>
       </c>
     </row>
     <row r="392" spans="1:4">
@@ -7654,7 +7597,7 @@
         <v>7</v>
       </c>
       <c r="D392" t="s">
-        <v>543</v>
+        <v>523</v>
       </c>
     </row>
     <row r="393" spans="1:4">
@@ -7668,7 +7611,7 @@
         <v>8</v>
       </c>
       <c r="D393" t="s">
-        <v>544</v>
+        <v>524</v>
       </c>
     </row>
     <row r="394" spans="1:4">
@@ -7682,7 +7625,7 @@
         <v>9</v>
       </c>
       <c r="D394" t="s">
-        <v>545</v>
+        <v>525</v>
       </c>
     </row>
     <row r="395" spans="1:4">
@@ -7696,7 +7639,7 @@
         <v>0</v>
       </c>
       <c r="D395" t="s">
-        <v>425</v>
+        <v>405</v>
       </c>
     </row>
     <row r="396" spans="1:4">
@@ -7710,7 +7653,7 @@
         <v>1</v>
       </c>
       <c r="D396" t="s">
-        <v>426</v>
+        <v>406</v>
       </c>
     </row>
     <row r="397" spans="1:4">
@@ -7724,7 +7667,7 @@
         <v>0</v>
       </c>
       <c r="D397" t="s">
-        <v>427</v>
+        <v>407</v>
       </c>
     </row>
     <row r="398" spans="1:4">
@@ -7738,7 +7681,7 @@
         <v>1</v>
       </c>
       <c r="D398" t="s">
-        <v>428</v>
+        <v>408</v>
       </c>
     </row>
     <row r="399" spans="1:4">
@@ -7752,7 +7695,7 @@
         <v>2</v>
       </c>
       <c r="D399" t="s">
-        <v>429</v>
+        <v>409</v>
       </c>
     </row>
     <row r="400" spans="1:4">
@@ -7766,7 +7709,7 @@
         <v>3</v>
       </c>
       <c r="D400" t="s">
-        <v>430</v>
+        <v>410</v>
       </c>
     </row>
     <row r="401" spans="1:4">
@@ -7780,7 +7723,7 @@
         <v>4</v>
       </c>
       <c r="D401" t="s">
-        <v>431</v>
+        <v>411</v>
       </c>
     </row>
     <row r="402" spans="1:4">
@@ -7794,7 +7737,7 @@
         <v>5</v>
       </c>
       <c r="D402" t="s">
-        <v>432</v>
+        <v>412</v>
       </c>
     </row>
     <row r="403" spans="1:4">
@@ -7808,7 +7751,7 @@
         <v>6</v>
       </c>
       <c r="D403" t="s">
-        <v>433</v>
+        <v>413</v>
       </c>
     </row>
     <row r="404" spans="1:4">
@@ -7822,7 +7765,7 @@
         <v>7</v>
       </c>
       <c r="D404" t="s">
-        <v>434</v>
+        <v>414</v>
       </c>
     </row>
     <row r="405" spans="1:4">
@@ -7836,7 +7779,7 @@
         <v>8</v>
       </c>
       <c r="D405" t="s">
-        <v>435</v>
+        <v>415</v>
       </c>
     </row>
     <row r="406" spans="1:4">
@@ -7850,7 +7793,7 @@
         <v>9</v>
       </c>
       <c r="D406" t="s">
-        <v>436</v>
+        <v>416</v>
       </c>
     </row>
     <row r="407" spans="1:4">
@@ -7864,7 +7807,7 @@
         <v>10</v>
       </c>
       <c r="D407" t="s">
-        <v>437</v>
+        <v>417</v>
       </c>
     </row>
     <row r="408" spans="1:4">
@@ -7878,7 +7821,7 @@
         <v>11</v>
       </c>
       <c r="D408" t="s">
-        <v>438</v>
+        <v>418</v>
       </c>
     </row>
     <row r="409" spans="1:4">
@@ -7892,7 +7835,7 @@
         <v>12</v>
       </c>
       <c r="D409" t="s">
-        <v>439</v>
+        <v>419</v>
       </c>
     </row>
     <row r="410" spans="1:4">
@@ -7906,7 +7849,7 @@
         <v>13</v>
       </c>
       <c r="D410" t="s">
-        <v>440</v>
+        <v>420</v>
       </c>
     </row>
     <row r="411" spans="1:4">
@@ -7920,7 +7863,7 @@
         <v>14</v>
       </c>
       <c r="D411" t="s">
-        <v>441</v>
+        <v>421</v>
       </c>
     </row>
     <row r="412" spans="1:4">
@@ -7934,7 +7877,7 @@
         <v>15</v>
       </c>
       <c r="D412" t="s">
-        <v>442</v>
+        <v>422</v>
       </c>
     </row>
     <row r="413" spans="1:4">
@@ -7948,7 +7891,7 @@
         <v>16</v>
       </c>
       <c r="D413" t="s">
-        <v>443</v>
+        <v>423</v>
       </c>
     </row>
     <row r="414" spans="1:4">
@@ -7962,7 +7905,7 @@
         <v>17</v>
       </c>
       <c r="D414" t="s">
-        <v>444</v>
+        <v>424</v>
       </c>
     </row>
     <row r="415" spans="1:4">
@@ -7976,7 +7919,7 @@
         <v>18</v>
       </c>
       <c r="D415" t="s">
-        <v>445</v>
+        <v>425</v>
       </c>
     </row>
     <row r="416" spans="1:4">
@@ -7990,7 +7933,7 @@
         <v>19</v>
       </c>
       <c r="D416" t="s">
-        <v>446</v>
+        <v>426</v>
       </c>
     </row>
     <row r="417" spans="1:4">
@@ -8004,7 +7947,7 @@
         <v>20</v>
       </c>
       <c r="D417" t="s">
-        <v>447</v>
+        <v>427</v>
       </c>
     </row>
     <row r="418" spans="1:4">
@@ -8018,7 +7961,7 @@
         <v>21</v>
       </c>
       <c r="D418" t="s">
-        <v>448</v>
+        <v>428</v>
       </c>
     </row>
     <row r="419" spans="1:4">
@@ -8032,7 +7975,7 @@
         <v>22</v>
       </c>
       <c r="D419" t="s">
-        <v>449</v>
+        <v>429</v>
       </c>
     </row>
     <row r="420" spans="1:4">
@@ -8046,7 +7989,7 @@
         <v>23</v>
       </c>
       <c r="D420" t="s">
-        <v>450</v>
+        <v>430</v>
       </c>
     </row>
     <row r="421" spans="1:4">
@@ -8060,7 +8003,7 @@
         <v>24</v>
       </c>
       <c r="D421" t="s">
-        <v>451</v>
+        <v>431</v>
       </c>
     </row>
     <row r="422" spans="1:4">
@@ -8074,7 +8017,7 @@
         <v>25</v>
       </c>
       <c r="D422" t="s">
-        <v>452</v>
+        <v>432</v>
       </c>
     </row>
     <row r="423" spans="1:4">
@@ -8088,7 +8031,7 @@
         <v>26</v>
       </c>
       <c r="D423" t="s">
-        <v>453</v>
+        <v>433</v>
       </c>
     </row>
     <row r="424" spans="1:4">
@@ -8102,7 +8045,7 @@
         <v>27</v>
       </c>
       <c r="D424" t="s">
-        <v>454</v>
+        <v>434</v>
       </c>
     </row>
     <row r="425" spans="1:4">
@@ -8116,7 +8059,7 @@
         <v>28</v>
       </c>
       <c r="D425" t="s">
-        <v>455</v>
+        <v>435</v>
       </c>
     </row>
     <row r="426" spans="1:4">
@@ -8130,7 +8073,7 @@
         <v>29</v>
       </c>
       <c r="D426" t="s">
-        <v>456</v>
+        <v>436</v>
       </c>
     </row>
     <row r="427" spans="1:4">
@@ -8144,7 +8087,7 @@
         <v>30</v>
       </c>
       <c r="D427" t="s">
-        <v>457</v>
+        <v>437</v>
       </c>
     </row>
     <row r="428" spans="1:4">
@@ -8158,7 +8101,7 @@
         <v>31</v>
       </c>
       <c r="D428" t="s">
-        <v>458</v>
+        <v>438</v>
       </c>
     </row>
     <row r="429" spans="1:4">
@@ -8172,7 +8115,7 @@
         <v>32</v>
       </c>
       <c r="D429" t="s">
-        <v>459</v>
+        <v>439</v>
       </c>
     </row>
     <row r="430" spans="1:4">
@@ -8186,7 +8129,7 @@
         <v>33</v>
       </c>
       <c r="D430" t="s">
-        <v>460</v>
+        <v>440</v>
       </c>
     </row>
     <row r="431" spans="1:4">
@@ -8200,7 +8143,7 @@
         <v>34</v>
       </c>
       <c r="D431" t="s">
-        <v>461</v>
+        <v>441</v>
       </c>
     </row>
     <row r="432" spans="1:4">
@@ -8214,7 +8157,7 @@
         <v>35</v>
       </c>
       <c r="D432" t="s">
-        <v>462</v>
+        <v>442</v>
       </c>
     </row>
     <row r="433" spans="1:4">
@@ -8228,7 +8171,7 @@
         <v>36</v>
       </c>
       <c r="D433" t="s">
-        <v>463</v>
+        <v>443</v>
       </c>
     </row>
     <row r="434" spans="1:4">
@@ -8242,7 +8185,7 @@
         <v>37</v>
       </c>
       <c r="D434" t="s">
-        <v>464</v>
+        <v>444</v>
       </c>
     </row>
     <row r="435" spans="1:4">
@@ -8256,7 +8199,7 @@
         <v>38</v>
       </c>
       <c r="D435" t="s">
-        <v>465</v>
+        <v>445</v>
       </c>
     </row>
     <row r="436" spans="1:4">
@@ -8270,7 +8213,7 @@
         <v>39</v>
       </c>
       <c r="D436" t="s">
-        <v>466</v>
+        <v>446</v>
       </c>
     </row>
     <row r="437" spans="1:4">
@@ -8284,7 +8227,7 @@
         <v>40</v>
       </c>
       <c r="D437" t="s">
-        <v>467</v>
+        <v>447</v>
       </c>
     </row>
     <row r="438" spans="1:4">
@@ -8298,7 +8241,7 @@
         <v>41</v>
       </c>
       <c r="D438" t="s">
-        <v>468</v>
+        <v>448</v>
       </c>
     </row>
     <row r="439" spans="1:4">
@@ -8312,7 +8255,7 @@
         <v>42</v>
       </c>
       <c r="D439" t="s">
-        <v>469</v>
+        <v>449</v>
       </c>
     </row>
     <row r="440" spans="1:4">
@@ -8326,7 +8269,7 @@
         <v>43</v>
       </c>
       <c r="D440" t="s">
-        <v>470</v>
+        <v>450</v>
       </c>
     </row>
     <row r="441" spans="1:4">
@@ -8340,7 +8283,7 @@
         <v>44</v>
       </c>
       <c r="D441" t="s">
-        <v>471</v>
+        <v>451</v>
       </c>
     </row>
     <row r="442" spans="1:4">
@@ -8354,7 +8297,7 @@
         <v>45</v>
       </c>
       <c r="D442" t="s">
-        <v>472</v>
+        <v>452</v>
       </c>
     </row>
     <row r="443" spans="1:4">
@@ -8368,7 +8311,7 @@
         <v>46</v>
       </c>
       <c r="D443" t="s">
-        <v>473</v>
+        <v>453</v>
       </c>
     </row>
     <row r="444" spans="1:4">
@@ -8382,7 +8325,7 @@
         <v>47</v>
       </c>
       <c r="D444" t="s">
-        <v>474</v>
+        <v>454</v>
       </c>
     </row>
     <row r="445" spans="1:4">
@@ -8396,7 +8339,7 @@
         <v>48</v>
       </c>
       <c r="D445" t="s">
-        <v>475</v>
+        <v>455</v>
       </c>
     </row>
     <row r="446" spans="1:4">
@@ -8410,7 +8353,7 @@
         <v>49</v>
       </c>
       <c r="D446" t="s">
-        <v>476</v>
+        <v>456</v>
       </c>
     </row>
     <row r="447" spans="1:4">
@@ -8424,7 +8367,7 @@
         <v>50</v>
       </c>
       <c r="D447" t="s">
-        <v>477</v>
+        <v>457</v>
       </c>
     </row>
     <row r="448" spans="1:4">
@@ -8438,7 +8381,7 @@
         <v>51</v>
       </c>
       <c r="D448" t="s">
-        <v>478</v>
+        <v>458</v>
       </c>
     </row>
     <row r="449" spans="1:4">
@@ -8452,7 +8395,7 @@
         <v>52</v>
       </c>
       <c r="D449" t="s">
-        <v>479</v>
+        <v>459</v>
       </c>
     </row>
     <row r="450" spans="1:4">
@@ -8466,7 +8409,7 @@
         <v>53</v>
       </c>
       <c r="D450" t="s">
-        <v>480</v>
+        <v>460</v>
       </c>
     </row>
     <row r="451" spans="1:4">
@@ -8480,7 +8423,7 @@
         <v>54</v>
       </c>
       <c r="D451" t="s">
-        <v>481</v>
+        <v>461</v>
       </c>
     </row>
     <row r="452" spans="1:4">
@@ -8494,7 +8437,7 @@
         <v>55</v>
       </c>
       <c r="D452" t="s">
-        <v>482</v>
+        <v>462</v>
       </c>
     </row>
     <row r="453" spans="1:4">
@@ -8508,7 +8451,7 @@
         <v>56</v>
       </c>
       <c r="D453" t="s">
-        <v>483</v>
+        <v>463</v>
       </c>
     </row>
     <row r="454" spans="1:4">
@@ -8522,7 +8465,7 @@
         <v>57</v>
       </c>
       <c r="D454" t="s">
-        <v>484</v>
+        <v>464</v>
       </c>
     </row>
     <row r="455" spans="1:4">
@@ -8536,7 +8479,7 @@
         <v>58</v>
       </c>
       <c r="D455" t="s">
-        <v>485</v>
+        <v>465</v>
       </c>
     </row>
     <row r="456" spans="1:4">
@@ -8550,7 +8493,7 @@
         <v>59</v>
       </c>
       <c r="D456" t="s">
-        <v>486</v>
+        <v>466</v>
       </c>
     </row>
     <row r="457" spans="1:4">
@@ -8564,7 +8507,7 @@
         <v>60</v>
       </c>
       <c r="D457" t="s">
-        <v>487</v>
+        <v>467</v>
       </c>
     </row>
     <row r="458" spans="1:4">
@@ -8578,7 +8521,7 @@
         <v>61</v>
       </c>
       <c r="D458" t="s">
-        <v>488</v>
+        <v>468</v>
       </c>
     </row>
     <row r="459" spans="1:4">
@@ -8592,7 +8535,7 @@
         <v>62</v>
       </c>
       <c r="D459" t="s">
-        <v>489</v>
+        <v>469</v>
       </c>
     </row>
     <row r="460" spans="1:4">
@@ -8606,7 +8549,7 @@
         <v>63</v>
       </c>
       <c r="D460" t="s">
-        <v>490</v>
+        <v>470</v>
       </c>
     </row>
     <row r="461" spans="1:4">
@@ -8620,7 +8563,7 @@
         <v>64</v>
       </c>
       <c r="D461" t="s">
-        <v>491</v>
+        <v>471</v>
       </c>
     </row>
     <row r="462" spans="1:4">
@@ -8634,7 +8577,7 @@
         <v>65</v>
       </c>
       <c r="D462" t="s">
-        <v>492</v>
+        <v>472</v>
       </c>
     </row>
     <row r="463" spans="1:4">
@@ -8648,7 +8591,7 @@
         <v>66</v>
       </c>
       <c r="D463" t="s">
-        <v>493</v>
+        <v>473</v>
       </c>
     </row>
     <row r="464" spans="1:4">
@@ -8662,7 +8605,7 @@
         <v>67</v>
       </c>
       <c r="D464" t="s">
-        <v>494</v>
+        <v>474</v>
       </c>
     </row>
     <row r="465" spans="1:4">
@@ -8676,7 +8619,7 @@
         <v>68</v>
       </c>
       <c r="D465" t="s">
-        <v>495</v>
+        <v>475</v>
       </c>
     </row>
     <row r="466" spans="1:4">
@@ -8690,7 +8633,7 @@
         <v>69</v>
       </c>
       <c r="D466" t="s">
-        <v>496</v>
+        <v>476</v>
       </c>
     </row>
     <row r="467" spans="1:4">
@@ -8704,7 +8647,7 @@
         <v>70</v>
       </c>
       <c r="D467" t="s">
-        <v>497</v>
+        <v>477</v>
       </c>
     </row>
     <row r="468" spans="1:4">
@@ -8718,7 +8661,7 @@
         <v>71</v>
       </c>
       <c r="D468" t="s">
-        <v>498</v>
+        <v>478</v>
       </c>
     </row>
     <row r="469" spans="1:4">
@@ -8732,7 +8675,7 @@
         <v>72</v>
       </c>
       <c r="D469" t="s">
-        <v>499</v>
+        <v>479</v>
       </c>
     </row>
     <row r="470" spans="1:4">
@@ -8746,7 +8689,7 @@
         <v>73</v>
       </c>
       <c r="D470" t="s">
-        <v>500</v>
+        <v>480</v>
       </c>
     </row>
     <row r="471" spans="1:4">
@@ -8760,7 +8703,7 @@
         <v>74</v>
       </c>
       <c r="D471" t="s">
-        <v>501</v>
+        <v>481</v>
       </c>
     </row>
     <row r="472" spans="1:4">
@@ -8774,7 +8717,7 @@
         <v>75</v>
       </c>
       <c r="D472" t="s">
-        <v>502</v>
+        <v>482</v>
       </c>
     </row>
     <row r="473" spans="1:4">
@@ -8788,7 +8731,7 @@
         <v>76</v>
       </c>
       <c r="D473" t="s">
-        <v>503</v>
+        <v>483</v>
       </c>
     </row>
     <row r="474" spans="1:4">
@@ -8802,7 +8745,7 @@
         <v>77</v>
       </c>
       <c r="D474" t="s">
-        <v>504</v>
+        <v>484</v>
       </c>
     </row>
     <row r="475" spans="1:4">
@@ -8816,7 +8759,7 @@
         <v>78</v>
       </c>
       <c r="D475" t="s">
-        <v>505</v>
+        <v>485</v>
       </c>
     </row>
     <row r="476" spans="1:4">
@@ -8830,7 +8773,7 @@
         <v>79</v>
       </c>
       <c r="D476" t="s">
-        <v>506</v>
+        <v>486</v>
       </c>
     </row>
     <row r="477" spans="1:4">
@@ -8844,7 +8787,7 @@
         <v>80</v>
       </c>
       <c r="D477" t="s">
-        <v>507</v>
+        <v>487</v>
       </c>
     </row>
     <row r="478" spans="1:4">
@@ -8858,7 +8801,7 @@
         <v>81</v>
       </c>
       <c r="D478" t="s">
-        <v>508</v>
+        <v>488</v>
       </c>
     </row>
     <row r="479" spans="1:4">
@@ -8872,7 +8815,7 @@
         <v>82</v>
       </c>
       <c r="D479" t="s">
-        <v>509</v>
+        <v>489</v>
       </c>
     </row>
     <row r="480" spans="1:4">
@@ -8886,7 +8829,7 @@
         <v>83</v>
       </c>
       <c r="D480" t="s">
-        <v>510</v>
+        <v>490</v>
       </c>
     </row>
     <row r="481" spans="1:4">
@@ -8900,7 +8843,7 @@
         <v>84</v>
       </c>
       <c r="D481" t="s">
-        <v>511</v>
+        <v>491</v>
       </c>
     </row>
     <row r="482" spans="1:4">
@@ -8914,7 +8857,7 @@
         <v>85</v>
       </c>
       <c r="D482" t="s">
-        <v>512</v>
+        <v>492</v>
       </c>
     </row>
     <row r="483" spans="1:4">
@@ -8928,7 +8871,7 @@
         <v>86</v>
       </c>
       <c r="D483" t="s">
-        <v>513</v>
+        <v>493</v>
       </c>
     </row>
     <row r="484" spans="1:4">
@@ -8942,7 +8885,7 @@
         <v>87</v>
       </c>
       <c r="D484" t="s">
-        <v>514</v>
+        <v>494</v>
       </c>
     </row>
     <row r="485" spans="1:4">
@@ -8956,7 +8899,7 @@
         <v>88</v>
       </c>
       <c r="D485" t="s">
-        <v>515</v>
+        <v>495</v>
       </c>
     </row>
     <row r="486" spans="1:4">
@@ -8970,7 +8913,7 @@
         <v>89</v>
       </c>
       <c r="D486" t="s">
-        <v>516</v>
+        <v>496</v>
       </c>
     </row>
     <row r="487" spans="1:4">
@@ -8984,7 +8927,7 @@
         <v>90</v>
       </c>
       <c r="D487" t="s">
-        <v>517</v>
+        <v>497</v>
       </c>
     </row>
     <row r="488" spans="1:4">
@@ -8998,7 +8941,7 @@
         <v>91</v>
       </c>
       <c r="D488" t="s">
-        <v>518</v>
+        <v>498</v>
       </c>
     </row>
     <row r="489" spans="1:4">
@@ -9012,7 +8955,7 @@
         <v>92</v>
       </c>
       <c r="D489" t="s">
-        <v>519</v>
+        <v>499</v>
       </c>
     </row>
     <row r="490" spans="1:4">
@@ -9026,7 +8969,7 @@
         <v>93</v>
       </c>
       <c r="D490" t="s">
-        <v>520</v>
+        <v>500</v>
       </c>
     </row>
     <row r="491" spans="1:4">
@@ -9040,7 +8983,7 @@
         <v>94</v>
       </c>
       <c r="D491" t="s">
-        <v>521</v>
+        <v>501</v>
       </c>
     </row>
     <row r="492" spans="1:4">
@@ -9054,7 +8997,7 @@
         <v>95</v>
       </c>
       <c r="D492" t="s">
-        <v>522</v>
+        <v>502</v>
       </c>
     </row>
     <row r="493" spans="1:4">
@@ -9068,7 +9011,7 @@
         <v>96</v>
       </c>
       <c r="D493" t="s">
-        <v>523</v>
+        <v>503</v>
       </c>
     </row>
     <row r="494" spans="1:4">
@@ -9082,7 +9025,7 @@
         <v>97</v>
       </c>
       <c r="D494" t="s">
-        <v>524</v>
+        <v>504</v>
       </c>
     </row>
     <row r="495" spans="1:4">
@@ -9096,7 +9039,7 @@
         <v>98</v>
       </c>
       <c r="D495" t="s">
-        <v>525</v>
+        <v>505</v>
       </c>
     </row>
     <row r="496" spans="1:4">
@@ -9110,7 +9053,7 @@
         <v>99</v>
       </c>
       <c r="D496" t="s">
-        <v>526</v>
+        <v>506</v>
       </c>
     </row>
     <row r="497" spans="1:4">
@@ -9124,7 +9067,7 @@
         <v>0</v>
       </c>
       <c r="D497" t="s">
-        <v>527</v>
+        <v>507</v>
       </c>
     </row>
     <row r="498" spans="1:4">
@@ -9138,7 +9081,7 @@
         <v>1</v>
       </c>
       <c r="D498" t="s">
-        <v>528</v>
+        <v>508</v>
       </c>
     </row>
     <row r="499" spans="1:4">
@@ -9152,7 +9095,7 @@
         <v>2</v>
       </c>
       <c r="D499" t="s">
-        <v>529</v>
+        <v>509</v>
       </c>
     </row>
     <row r="500" spans="1:4">
@@ -9166,7 +9109,7 @@
         <v>3</v>
       </c>
       <c r="D500" t="s">
-        <v>534</v>
+        <v>514</v>
       </c>
     </row>
     <row r="501" spans="1:4">
@@ -9180,7 +9123,7 @@
         <v>4</v>
       </c>
       <c r="D501" t="s">
-        <v>533</v>
+        <v>513</v>
       </c>
     </row>
     <row r="502" spans="1:4">
@@ -9194,7 +9137,7 @@
         <v>5</v>
       </c>
       <c r="D502" t="s">
-        <v>535</v>
+        <v>515</v>
       </c>
     </row>
     <row r="503" spans="1:4">
@@ -9208,7 +9151,7 @@
         <v>6</v>
       </c>
       <c r="D503" t="s">
-        <v>532</v>
+        <v>512</v>
       </c>
     </row>
     <row r="504" spans="1:4">
@@ -9222,7 +9165,7 @@
         <v>7</v>
       </c>
       <c r="D504" t="s">
-        <v>530</v>
+        <v>510</v>
       </c>
     </row>
     <row r="505" spans="1:4">
@@ -9236,7 +9179,7 @@
         <v>8</v>
       </c>
       <c r="D505" t="s">
-        <v>531</v>
+        <v>511</v>
       </c>
     </row>
     <row r="506" spans="1:4">
@@ -9250,7 +9193,7 @@
         <v>0</v>
       </c>
       <c r="D506" t="s">
-        <v>537</v>
+        <v>517</v>
       </c>
     </row>
     <row r="507" spans="1:4">
@@ -9264,7 +9207,7 @@
         <v>1</v>
       </c>
       <c r="D507" t="s">
-        <v>536</v>
+        <v>516</v>
       </c>
     </row>
   </sheetData>

</xml_diff>